<commit_message>
ADD REL IN 30 MIN
</commit_message>
<xml_diff>
--- a/cash high low.xlsx
+++ b/cash high low.xlsx
@@ -642,22 +642,22 @@
         </is>
       </c>
       <c r="B2" s="8" t="n">
-        <v>526.45</v>
+        <v>514.8</v>
       </c>
       <c r="C2" s="11" t="n">
-        <v>509.05</v>
+        <v>504.5</v>
       </c>
       <c r="D2" s="14" t="n">
-        <v>523</v>
+        <v>512</v>
       </c>
       <c r="E2" s="5" t="n">
-        <v>524.25</v>
+        <v>510.9</v>
       </c>
       <c r="F2" s="17" t="n">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="G2" s="5" t="n">
-        <v>516.3</v>
+        <v>507.75</v>
       </c>
     </row>
     <row r="3">
@@ -667,22 +667,22 @@
         </is>
       </c>
       <c r="B3" s="8" t="n">
-        <v>3031.7</v>
+        <v>2976.5</v>
       </c>
       <c r="C3" s="11" t="n">
-        <v>2974.05</v>
+        <v>2933.85</v>
       </c>
       <c r="D3" s="14" t="n">
-        <v>2999.95</v>
+        <v>2948.95</v>
       </c>
       <c r="E3" s="5" t="n">
-        <v>3002</v>
+        <v>2947.25</v>
       </c>
       <c r="F3" s="17" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="G3" s="5" t="n">
-        <v>2979</v>
+        <v>2937.8</v>
       </c>
     </row>
     <row r="4">
@@ -692,22 +692,22 @@
         </is>
       </c>
       <c r="B4" s="9" t="n">
-        <v>510.9</v>
+        <v>508</v>
       </c>
       <c r="C4" s="12" t="n">
+        <v>497.25</v>
+      </c>
+      <c r="D4" s="15" t="n">
+        <v>502</v>
+      </c>
+      <c r="E4" s="6" t="n">
+        <v>504.95</v>
+      </c>
+      <c r="F4" s="18" t="n">
+        <v>10</v>
+      </c>
+      <c r="G4" s="6" t="n">
         <v>498.2</v>
-      </c>
-      <c r="D4" s="15" t="n">
-        <v>505.55</v>
-      </c>
-      <c r="E4" s="6" t="n">
-        <v>505.75</v>
-      </c>
-      <c r="F4" s="18" t="n">
-        <v>18</v>
-      </c>
-      <c r="G4" s="6" t="n">
-        <v>499.15</v>
       </c>
     </row>
     <row r="5">
@@ -717,22 +717,22 @@
         </is>
       </c>
       <c r="B5" s="9" t="n">
-        <v>1833.3</v>
+        <v>1755</v>
       </c>
       <c r="C5" s="12" t="n">
-        <v>1800</v>
+        <v>1725.05</v>
       </c>
       <c r="D5" s="15" t="n">
-        <v>1821.5</v>
+        <v>1748</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>1819.9</v>
+        <v>1750.75</v>
       </c>
       <c r="F5" s="18" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>1807</v>
+        <v>1742.85</v>
       </c>
     </row>
     <row r="6">
@@ -742,22 +742,22 @@
         </is>
       </c>
       <c r="B6" s="9" t="n">
-        <v>6938.65</v>
+        <v>6970.8</v>
       </c>
       <c r="C6" s="12" t="n">
-        <v>6820.7</v>
+        <v>6879.75</v>
       </c>
       <c r="D6" s="15" t="n">
-        <v>6910.05</v>
+        <v>6897.35</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>6899.55</v>
+        <v>6889.75</v>
       </c>
       <c r="F6" s="18" t="n">
         <v>7</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>6844.25</v>
+        <v>6918</v>
       </c>
     </row>
     <row r="7">
@@ -767,22 +767,22 @@
         </is>
       </c>
       <c r="B7" s="9" t="n">
-        <v>192.68</v>
+        <v>183.25</v>
       </c>
       <c r="C7" s="12" t="n">
-        <v>188.68</v>
+        <v>176.77</v>
       </c>
       <c r="D7" s="15" t="n">
-        <v>191.96</v>
+        <v>182.5</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>191.96</v>
+        <v>182.21</v>
       </c>
       <c r="F7" s="18" t="n">
-        <v>98</v>
+        <v>169</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>188.9</v>
+        <v>177.4</v>
       </c>
     </row>
     <row r="8">
@@ -792,22 +792,22 @@
         </is>
       </c>
       <c r="B8" s="9" t="n">
-        <v>248.75</v>
+        <v>254.18</v>
       </c>
       <c r="C8" s="12" t="n">
-        <v>237.85</v>
+        <v>248.2</v>
       </c>
       <c r="D8" s="15" t="n">
-        <v>247.5</v>
+        <v>252.25</v>
       </c>
       <c r="E8" s="6" t="n">
-        <v>247.97</v>
+        <v>250.96</v>
       </c>
       <c r="F8" s="18" t="n">
-        <v>109</v>
+        <v>77</v>
       </c>
       <c r="G8" s="6" t="n">
-        <v>238.2</v>
+        <v>251.85</v>
       </c>
     </row>
     <row r="9">
@@ -817,22 +817,22 @@
         </is>
       </c>
       <c r="B9" s="9" t="n">
-        <v>493.75</v>
+        <v>454.5</v>
       </c>
       <c r="C9" s="12" t="n">
-        <v>483.35</v>
+        <v>443.2</v>
       </c>
       <c r="D9" s="15" t="n">
-        <v>491.05</v>
+        <v>452.55</v>
       </c>
       <c r="E9" s="6" t="n">
-        <v>492.2</v>
+        <v>452.05</v>
       </c>
       <c r="F9" s="18" t="n">
-        <v>45</v>
+        <v>84</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>484.7</v>
+        <v>444.65</v>
       </c>
     </row>
     <row r="10">
@@ -842,22 +842,22 @@
         </is>
       </c>
       <c r="B10" s="9" t="n">
-        <v>880.35</v>
+        <v>828.7</v>
       </c>
       <c r="C10" s="12" t="n">
-        <v>848.7</v>
+        <v>814.3</v>
       </c>
       <c r="D10" s="15" t="n">
-        <v>874</v>
+        <v>819.7</v>
       </c>
       <c r="E10" s="6" t="n">
-        <v>875.15</v>
+        <v>819.85</v>
       </c>
       <c r="F10" s="18" t="n">
         <v>24</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>851.25</v>
+        <v>824.6</v>
       </c>
     </row>
     <row r="11">
@@ -867,22 +867,22 @@
         </is>
       </c>
       <c r="B11" s="9" t="n">
-        <v>4799.9</v>
+        <v>4915</v>
       </c>
       <c r="C11" s="12" t="n">
-        <v>4670.6</v>
+        <v>4820.7</v>
       </c>
       <c r="D11" s="15" t="n">
-        <v>4761.75</v>
+        <v>4909.95</v>
       </c>
       <c r="E11" s="6" t="n">
-        <v>4765.65</v>
+        <v>4894.65</v>
       </c>
       <c r="F11" s="18" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>4691.6</v>
+        <v>4851.55</v>
       </c>
     </row>
     <row r="12">
@@ -892,22 +892,22 @@
         </is>
       </c>
       <c r="B12" s="9" t="n">
-        <v>196.25</v>
+        <v>205.66</v>
       </c>
       <c r="C12" s="12" t="n">
-        <v>190.59</v>
+        <v>201.02</v>
       </c>
       <c r="D12" s="15" t="n">
-        <v>195.05</v>
+        <v>204.29</v>
       </c>
       <c r="E12" s="6" t="n">
-        <v>195.3</v>
+        <v>203.91</v>
       </c>
       <c r="F12" s="18" t="n">
-        <v>73</v>
+        <v>130</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>190.86</v>
+        <v>203.02</v>
       </c>
     </row>
     <row r="13">
@@ -917,22 +917,22 @@
         </is>
       </c>
       <c r="B13" s="9" t="n">
-        <v>1870.5</v>
+        <v>1819.9</v>
       </c>
       <c r="C13" s="12" t="n">
-        <v>1843</v>
+        <v>1756.55</v>
       </c>
       <c r="D13" s="15" t="n">
-        <v>1856.55</v>
+        <v>1772.5</v>
       </c>
       <c r="E13" s="6" t="n">
-        <v>1857.7</v>
+        <v>1766.05</v>
       </c>
       <c r="F13" s="18" t="n">
-        <v>23</v>
+        <v>36</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>1862.95</v>
+        <v>1817.3</v>
       </c>
     </row>
     <row r="14">
@@ -942,22 +942,22 @@
         </is>
       </c>
       <c r="B14" s="9" t="n">
-        <v>1691</v>
+        <v>1738.9</v>
       </c>
       <c r="C14" s="12" t="n">
-        <v>1654.1</v>
+        <v>1719.4</v>
       </c>
       <c r="D14" s="15" t="n">
-        <v>1684.8</v>
+        <v>1734.3</v>
       </c>
       <c r="E14" s="6" t="n">
-        <v>1681.85</v>
+        <v>1735.7</v>
       </c>
       <c r="F14" s="18" t="n">
-        <v>124</v>
+        <v>114</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>1655.7</v>
+        <v>1728.3</v>
       </c>
     </row>
     <row r="15">
@@ -967,22 +967,22 @@
         </is>
       </c>
       <c r="B15" s="9" t="n">
-        <v>756.45</v>
+        <v>689.55</v>
       </c>
       <c r="C15" s="12" t="n">
-        <v>725.5</v>
+        <v>679.25</v>
       </c>
       <c r="D15" s="15" t="n">
-        <v>753.2</v>
+        <v>684.1</v>
       </c>
       <c r="E15" s="6" t="n">
-        <v>753.5</v>
+        <v>686.05</v>
       </c>
       <c r="F15" s="18" t="n">
-        <v>54</v>
+        <v>44</v>
       </c>
       <c r="G15" s="6" t="n">
-        <v>725.6</v>
+        <v>685.4</v>
       </c>
     </row>
     <row r="16">
@@ -992,22 +992,22 @@
         </is>
       </c>
       <c r="B16" s="9" t="n">
-        <v>1268.9</v>
+        <v>1316.65</v>
       </c>
       <c r="C16" s="12" t="n">
-        <v>1225.75</v>
+        <v>1288.55</v>
       </c>
       <c r="D16" s="15" t="n">
-        <v>1267</v>
+        <v>1294.8</v>
       </c>
       <c r="E16" s="6" t="n">
-        <v>1264.5</v>
+        <v>1292.25</v>
       </c>
       <c r="F16" s="18" t="n">
-        <v>110</v>
+        <v>234</v>
       </c>
       <c r="G16" s="6" t="n">
-        <v>1228.55</v>
+        <v>1314.95</v>
       </c>
     </row>
     <row r="17">
@@ -1017,22 +1017,22 @@
         </is>
       </c>
       <c r="B17" s="9" t="n">
-        <v>1354.95</v>
+        <v>1066.9</v>
       </c>
       <c r="C17" s="12" t="n">
-        <v>1331.5</v>
+        <v>1044</v>
       </c>
       <c r="D17" s="15" t="n">
-        <v>1347.95</v>
+        <v>1055</v>
       </c>
       <c r="E17" s="6" t="n">
-        <v>1347.25</v>
+        <v>1055.6</v>
       </c>
       <c r="F17" s="18" t="n">
-        <v>36</v>
+        <v>45</v>
       </c>
       <c r="G17" s="6" t="n">
-        <v>1333.85</v>
+        <v>1050.4</v>
       </c>
     </row>
     <row r="18">
@@ -1042,22 +1042,22 @@
         </is>
       </c>
       <c r="B18" s="9" t="n">
-        <v>1936.85</v>
+        <v>1771</v>
       </c>
       <c r="C18" s="12" t="n">
-        <v>1869.25</v>
+        <v>1746.5</v>
       </c>
       <c r="D18" s="15" t="n">
-        <v>1885</v>
+        <v>1762.95</v>
       </c>
       <c r="E18" s="6" t="n">
-        <v>1879.6</v>
+        <v>1757.25</v>
       </c>
       <c r="F18" s="18" t="n">
-        <v>105</v>
+        <v>73</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>1930</v>
+        <v>1768.9</v>
       </c>
     </row>
     <row r="19">
@@ -1067,22 +1067,22 @@
         </is>
       </c>
       <c r="B19" s="9" t="n">
-        <v>973.2</v>
+        <v>931.7</v>
       </c>
       <c r="C19" s="12" t="n">
-        <v>923.7</v>
+        <v>911.55</v>
       </c>
       <c r="D19" s="15" t="n">
-        <v>965</v>
+        <v>919</v>
       </c>
       <c r="E19" s="6" t="n">
-        <v>964.5</v>
+        <v>920.5</v>
       </c>
       <c r="F19" s="18" t="n">
-        <v>26</v>
+        <v>11</v>
       </c>
       <c r="G19" s="6" t="n">
-        <v>924</v>
+        <v>922.5</v>
       </c>
     </row>
     <row r="20">
@@ -1092,22 +1092,22 @@
         </is>
       </c>
       <c r="B20" s="9" t="n">
-        <v>619.9</v>
+        <v>635.45</v>
       </c>
       <c r="C20" s="12" t="n">
-        <v>602.25</v>
+        <v>621.45</v>
       </c>
       <c r="D20" s="15" t="n">
-        <v>619.6</v>
+        <v>632</v>
       </c>
       <c r="E20" s="6" t="n">
-        <v>618.6</v>
+        <v>631.05</v>
       </c>
       <c r="F20" s="18" t="n">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="G20" s="6" t="n">
-        <v>602.55</v>
+        <v>630.2</v>
       </c>
     </row>
     <row r="21">
@@ -1117,22 +1117,22 @@
         </is>
       </c>
       <c r="B21" s="9" t="n">
-        <v>2988.85</v>
+        <v>2752</v>
       </c>
       <c r="C21" s="12" t="n">
-        <v>2928</v>
+        <v>2671.6</v>
       </c>
       <c r="D21" s="15" t="n">
-        <v>2965</v>
+        <v>2751.3</v>
       </c>
       <c r="E21" s="6" t="n">
-        <v>2964.25</v>
+        <v>2728.55</v>
       </c>
       <c r="F21" s="18" t="n">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="G21" s="6" t="n">
-        <v>2940.75</v>
+        <v>2692.95</v>
       </c>
     </row>
     <row r="22">
@@ -1142,22 +1142,22 @@
         </is>
       </c>
       <c r="B22" s="9" t="n">
-        <v>293.4</v>
+        <v>274.55</v>
       </c>
       <c r="C22" s="12" t="n">
-        <v>280</v>
+        <v>266.7</v>
       </c>
       <c r="D22" s="15" t="n">
-        <v>291.1</v>
+        <v>269.8</v>
       </c>
       <c r="E22" s="6" t="n">
-        <v>291</v>
+        <v>270.6</v>
       </c>
       <c r="F22" s="18" t="n">
-        <v>34</v>
+        <v>26</v>
       </c>
       <c r="G22" s="6" t="n">
-        <v>280.5</v>
+        <v>274.2</v>
       </c>
     </row>
     <row r="23">
@@ -1167,22 +1167,22 @@
         </is>
       </c>
       <c r="B23" s="9" t="n">
-        <v>425.95</v>
+        <v>410.65</v>
       </c>
       <c r="C23" s="12" t="n">
-        <v>414.85</v>
+        <v>403.5</v>
       </c>
       <c r="D23" s="15" t="n">
-        <v>425.1</v>
+        <v>408.3</v>
       </c>
       <c r="E23" s="6" t="n">
-        <v>424.95</v>
+        <v>408.15</v>
       </c>
       <c r="F23" s="18" t="n">
-        <v>88</v>
+        <v>122</v>
       </c>
       <c r="G23" s="6" t="n">
-        <v>414.95</v>
+        <v>404.4</v>
       </c>
     </row>
     <row r="24">
@@ -1192,22 +1192,22 @@
         </is>
       </c>
       <c r="B24" s="9" t="n">
-        <v>2736.85</v>
+        <v>1340.9</v>
       </c>
       <c r="C24" s="12" t="n">
-        <v>2682.65</v>
+        <v>1326.15</v>
       </c>
       <c r="D24" s="15" t="n">
-        <v>2717</v>
+        <v>1332</v>
       </c>
       <c r="E24" s="6" t="n">
-        <v>2718.6</v>
+        <v>1332.05</v>
       </c>
       <c r="F24" s="18" t="n">
-        <v>60</v>
+        <v>93</v>
       </c>
       <c r="G24" s="6" t="n">
-        <v>2684.1</v>
+        <v>1336.95</v>
       </c>
     </row>
     <row r="25">
@@ -1217,22 +1217,22 @@
         </is>
       </c>
       <c r="B25" s="9" t="n">
-        <v>822.6</v>
+        <v>828</v>
       </c>
       <c r="C25" s="12" t="n">
-        <v>802.9</v>
+        <v>813.55</v>
       </c>
       <c r="D25" s="15" t="n">
-        <v>819.95</v>
+        <v>821.1</v>
       </c>
       <c r="E25" s="6" t="n">
-        <v>820.4</v>
+        <v>820.2</v>
       </c>
       <c r="F25" s="18" t="n">
-        <v>117</v>
+        <v>134</v>
       </c>
       <c r="G25" s="6" t="n">
-        <v>804.95</v>
+        <v>822.65</v>
       </c>
     </row>
     <row r="26">
@@ -1242,22 +1242,22 @@
         </is>
       </c>
       <c r="B26" s="9" t="n">
-        <v>763.95</v>
+        <v>765</v>
       </c>
       <c r="C26" s="12" t="n">
-        <v>757</v>
+        <v>734.2</v>
       </c>
       <c r="D26" s="15" t="n">
-        <v>759.15</v>
+        <v>764.1</v>
       </c>
       <c r="E26" s="6" t="n">
-        <v>759.95</v>
+        <v>752.2</v>
       </c>
       <c r="F26" s="18" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="G26" s="6" t="n">
-        <v>757.3</v>
+        <v>744.15</v>
       </c>
     </row>
     <row r="27">
@@ -1267,22 +1267,22 @@
         </is>
       </c>
       <c r="B27" s="9" t="n">
-        <v>1093.45</v>
+        <v>1158.4</v>
       </c>
       <c r="C27" s="12" t="n">
-        <v>1040</v>
+        <v>1124.7</v>
       </c>
       <c r="D27" s="15" t="n">
-        <v>1083.95</v>
+        <v>1149</v>
       </c>
       <c r="E27" s="6" t="n">
-        <v>1088.1</v>
+        <v>1148.9</v>
       </c>
       <c r="F27" s="18" t="n">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="G27" s="6" t="n">
-        <v>1047.95</v>
+        <v>1128.8</v>
       </c>
     </row>
     <row r="28">
@@ -1292,22 +1292,22 @@
         </is>
       </c>
       <c r="B28" s="9" t="n">
-        <v>917.7</v>
+        <v>839.9</v>
       </c>
       <c r="C28" s="12" t="n">
-        <v>889.2</v>
+        <v>831.85</v>
       </c>
       <c r="D28" s="15" t="n">
-        <v>911</v>
+        <v>835.25</v>
       </c>
       <c r="E28" s="6" t="n">
-        <v>910.15</v>
+        <v>834.05</v>
       </c>
       <c r="F28" s="18" t="n">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="G28" s="6" t="n">
-        <v>890.5</v>
+        <v>835.4</v>
       </c>
     </row>
     <row r="29">
@@ -1317,22 +1317,22 @@
         </is>
       </c>
       <c r="B29" s="9" t="n">
-        <v>456.5</v>
+        <v>444.8</v>
       </c>
       <c r="C29" s="12" t="n">
-        <v>443.15</v>
+        <v>420.8</v>
       </c>
       <c r="D29" s="15" t="n">
-        <v>453.55</v>
+        <v>439.95</v>
       </c>
       <c r="E29" s="6" t="n">
-        <v>453.55</v>
+        <v>440.05</v>
       </c>
       <c r="F29" s="18" t="n">
-        <v>110</v>
+        <v>296</v>
       </c>
       <c r="G29" s="6" t="n">
-        <v>443.7</v>
+        <v>424.45</v>
       </c>
     </row>
     <row r="30">
@@ -1342,22 +1342,22 @@
         </is>
       </c>
       <c r="B30" s="9" t="n">
-        <v>156.2</v>
+        <v>149.95</v>
       </c>
       <c r="C30" s="12" t="n">
-        <v>151.1</v>
+        <v>148.24</v>
       </c>
       <c r="D30" s="15" t="n">
-        <v>155.5</v>
+        <v>148.33</v>
       </c>
       <c r="E30" s="6" t="n">
-        <v>155.39</v>
+        <v>148.56</v>
       </c>
       <c r="F30" s="18" t="n">
-        <v>347</v>
+        <v>263</v>
       </c>
       <c r="G30" s="6" t="n">
-        <v>151.16</v>
+        <v>149.07</v>
       </c>
     </row>
     <row r="31" ht="15.75" customHeight="1" thickBot="1">
@@ -1367,22 +1367,22 @@
         </is>
       </c>
       <c r="B31" s="10" t="n">
-        <v>11139.95</v>
+        <v>11250.9</v>
       </c>
       <c r="C31" s="13" t="n">
-        <v>10901</v>
+        <v>11042.55</v>
       </c>
       <c r="D31" s="16" t="n">
-        <v>11084</v>
+        <v>11076.9</v>
       </c>
       <c r="E31" s="7" t="n">
-        <v>11069.3</v>
+        <v>11065.65</v>
       </c>
       <c r="F31" s="19" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G31" s="7" t="n">
-        <v>10915.35</v>
+        <v>11115.2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fixed row nums for nifty and bn in 30 min csh
</commit_message>
<xml_diff>
--- a/cash high low.xlsx
+++ b/cash high low.xlsx
@@ -748,22 +748,22 @@
         </is>
       </c>
       <c r="B2" s="20" t="n">
-        <v>459.75</v>
+        <v>451.95</v>
       </c>
       <c r="C2" s="17" t="n">
-        <v>445.85</v>
+        <v>445.2</v>
       </c>
       <c r="D2" s="6" t="n">
-        <v>449.5</v>
+        <v>447.05</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>448.35</v>
+        <v>448.3</v>
       </c>
       <c r="F2" s="8" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>453.9</v>
+        <v>449.55</v>
       </c>
     </row>
     <row r="3">
@@ -773,22 +773,22 @@
         </is>
       </c>
       <c r="B3" s="20" t="n">
-        <v>2526.3</v>
+        <v>2520</v>
       </c>
       <c r="C3" s="17" t="n">
         <v>2400</v>
       </c>
       <c r="D3" s="6" t="n">
-        <v>2437</v>
+        <v>2457</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>2437.1</v>
+        <v>2463.15</v>
       </c>
       <c r="F3" s="8" t="n">
-        <v>144</v>
+        <v>81</v>
       </c>
       <c r="G3" s="4" t="n">
-        <v>2416.5</v>
+        <v>2470.9</v>
       </c>
     </row>
     <row r="4">
@@ -798,22 +798,22 @@
         </is>
       </c>
       <c r="B4" s="21" t="n">
-        <v>515</v>
+        <v>511.85</v>
       </c>
       <c r="C4" s="18" t="n">
-        <v>506.1</v>
+        <v>504.4</v>
       </c>
       <c r="D4" s="7" t="n">
-        <v>510</v>
+        <v>509.25</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>510.4</v>
+        <v>509.65</v>
       </c>
       <c r="F4" s="9" t="n">
         <v>8</v>
       </c>
       <c r="G4" s="5" t="n">
-        <v>511.9</v>
+        <v>506.75</v>
       </c>
     </row>
     <row r="5">
@@ -823,22 +823,22 @@
         </is>
       </c>
       <c r="B5" s="21" t="n">
-        <v>1598.15</v>
+        <v>1587.95</v>
       </c>
       <c r="C5" s="18" t="n">
-        <v>1567.65</v>
+        <v>1574.95</v>
       </c>
       <c r="D5" s="7" t="n">
-        <v>1582.3</v>
+        <v>1580</v>
       </c>
       <c r="E5" s="5" t="n">
-        <v>1575.05</v>
+        <v>1579.95</v>
       </c>
       <c r="F5" s="9" t="n">
-        <v>34</v>
+        <v>19</v>
       </c>
       <c r="G5" s="5" t="n">
-        <v>1596.5</v>
+        <v>1579</v>
       </c>
     </row>
     <row r="6">
@@ -848,22 +848,22 @@
         </is>
       </c>
       <c r="B6" s="21" t="n">
-        <v>6725</v>
+        <v>6609</v>
       </c>
       <c r="C6" s="18" t="n">
-        <v>6495</v>
+        <v>6510.35</v>
       </c>
       <c r="D6" s="7" t="n">
-        <v>6539</v>
+        <v>6565</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>6509.4</v>
+        <v>6575.9</v>
       </c>
       <c r="F6" s="9" t="n">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="G6" s="5" t="n">
-        <v>6664.15</v>
+        <v>6524.1</v>
       </c>
     </row>
     <row r="7">
@@ -873,22 +873,22 @@
         </is>
       </c>
       <c r="B7" s="21" t="n">
-        <v>174.07</v>
+        <v>171.58</v>
       </c>
       <c r="C7" s="18" t="n">
-        <v>170.3</v>
+        <v>167.12</v>
       </c>
       <c r="D7" s="7" t="n">
-        <v>171.49</v>
+        <v>168.94</v>
       </c>
       <c r="E7" s="5" t="n">
-        <v>170.96</v>
+        <v>169.08</v>
       </c>
       <c r="F7" s="9" t="n">
-        <v>80</v>
+        <v>88</v>
       </c>
       <c r="G7" s="5" t="n">
-        <v>171.88</v>
+        <v>171.1</v>
       </c>
     </row>
     <row r="8">
@@ -898,22 +898,22 @@
         </is>
       </c>
       <c r="B8" s="21" t="n">
-        <v>252</v>
+        <v>250.45</v>
       </c>
       <c r="C8" s="18" t="n">
-        <v>245.6</v>
+        <v>244.25</v>
       </c>
       <c r="D8" s="7" t="n">
-        <v>250.15</v>
+        <v>246.3</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>249</v>
+        <v>246.4</v>
       </c>
       <c r="F8" s="9" t="n">
-        <v>126</v>
+        <v>90</v>
       </c>
       <c r="G8" s="5" t="n">
-        <v>247</v>
+        <v>249.85</v>
       </c>
     </row>
     <row r="9">
@@ -923,22 +923,22 @@
         </is>
       </c>
       <c r="B9" s="21" t="n">
-        <v>424.9</v>
+        <v>418</v>
       </c>
       <c r="C9" s="18" t="n">
-        <v>413.5</v>
+        <v>411</v>
       </c>
       <c r="D9" s="7" t="n">
         <v>416.5</v>
       </c>
       <c r="E9" s="5" t="n">
-        <v>415.2</v>
+        <v>416.4</v>
       </c>
       <c r="F9" s="9" t="n">
-        <v>77</v>
+        <v>70</v>
       </c>
       <c r="G9" s="5" t="n">
-        <v>420.65</v>
+        <v>413.75</v>
       </c>
     </row>
     <row r="10">
@@ -948,22 +948,22 @@
         </is>
       </c>
       <c r="B10" s="21" t="n">
-        <v>826.4</v>
+        <v>828.65</v>
       </c>
       <c r="C10" s="18" t="n">
-        <v>808.95</v>
+        <v>813.05</v>
       </c>
       <c r="D10" s="7" t="n">
-        <v>815.4</v>
+        <v>822</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>813.85</v>
+        <v>822.95</v>
       </c>
       <c r="F10" s="9" t="n">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="G10" s="5" t="n">
-        <v>822.05</v>
+        <v>814.35</v>
       </c>
     </row>
     <row r="11">
@@ -973,22 +973,22 @@
         </is>
       </c>
       <c r="B11" s="21" t="n">
-        <v>4883.3</v>
+        <v>4864.3</v>
       </c>
       <c r="C11" s="18" t="n">
-        <v>4793.8</v>
+        <v>4808</v>
       </c>
       <c r="D11" s="7" t="n">
-        <v>4849</v>
+        <v>4832.2</v>
       </c>
       <c r="E11" s="5" t="n">
-        <v>4815.7</v>
+        <v>4831.85</v>
       </c>
       <c r="F11" s="9" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="G11" s="5" t="n">
-        <v>4877.75</v>
+        <v>4830.4</v>
       </c>
     </row>
     <row r="12">
@@ -998,22 +998,22 @@
         </is>
       </c>
       <c r="B12" s="21" t="n">
-        <v>212.7</v>
+        <v>211.49</v>
       </c>
       <c r="C12" s="18" t="n">
-        <v>210.4</v>
+        <v>208.79</v>
       </c>
       <c r="D12" s="7" t="n">
-        <v>211.24</v>
+        <v>210.79</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>211.05</v>
+        <v>210.78</v>
       </c>
       <c r="F12" s="9" t="n">
-        <v>109</v>
+        <v>72</v>
       </c>
       <c r="G12" s="5" t="n">
-        <v>211.86</v>
+        <v>210.36</v>
       </c>
     </row>
     <row r="13">
@@ -1023,22 +1023,22 @@
         </is>
       </c>
       <c r="B13" s="21" t="n">
-        <v>1883.25</v>
+        <v>1872.3</v>
       </c>
       <c r="C13" s="18" t="n">
-        <v>1835</v>
+        <v>1844.15</v>
       </c>
       <c r="D13" s="7" t="n">
-        <v>1844</v>
+        <v>1850</v>
       </c>
       <c r="E13" s="5" t="n">
-        <v>1840.9</v>
+        <v>1848.05</v>
       </c>
       <c r="F13" s="9" t="n">
-        <v>36</v>
+        <v>24</v>
       </c>
       <c r="G13" s="5" t="n">
-        <v>1878.6</v>
+        <v>1845.05</v>
       </c>
     </row>
     <row r="14">
@@ -1048,22 +1048,22 @@
         </is>
       </c>
       <c r="B14" s="21" t="n">
-        <v>1836.1</v>
+        <v>1802.8</v>
       </c>
       <c r="C14" s="18" t="n">
-        <v>1788</v>
+        <v>1782.9</v>
       </c>
       <c r="D14" s="7" t="n">
-        <v>1793</v>
+        <v>1795.5</v>
       </c>
       <c r="E14" s="5" t="n">
-        <v>1793.15</v>
+        <v>1796.05</v>
       </c>
       <c r="F14" s="9" t="n">
-        <v>178</v>
+        <v>138</v>
       </c>
       <c r="G14" s="5" t="n">
-        <v>1826.95</v>
+        <v>1795</v>
       </c>
     </row>
     <row r="15">
@@ -1073,22 +1073,22 @@
         </is>
       </c>
       <c r="B15" s="21" t="n">
-        <v>663.15</v>
+        <v>658.6</v>
       </c>
       <c r="C15" s="18" t="n">
-        <v>647.6</v>
+        <v>649.1</v>
       </c>
       <c r="D15" s="7" t="n">
-        <v>651.95</v>
+        <v>657</v>
       </c>
       <c r="E15" s="5" t="n">
-        <v>650.25</v>
+        <v>656.2</v>
       </c>
       <c r="F15" s="9" t="n">
-        <v>46</v>
+        <v>34</v>
       </c>
       <c r="G15" s="5" t="n">
-        <v>658.8</v>
+        <v>650.45</v>
       </c>
     </row>
     <row r="16">
@@ -1098,22 +1098,22 @@
         </is>
       </c>
       <c r="B16" s="21" t="n">
-        <v>1310.5</v>
+        <v>1303.25</v>
       </c>
       <c r="C16" s="18" t="n">
-        <v>1282.3</v>
+        <v>1287.6</v>
       </c>
       <c r="D16" s="7" t="n">
-        <v>1287.5</v>
+        <v>1298.7</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>1286.35</v>
+        <v>1300.1</v>
       </c>
       <c r="F16" s="9" t="n">
-        <v>228</v>
+        <v>113</v>
       </c>
       <c r="G16" s="5" t="n">
-        <v>1301.75</v>
+        <v>1291.25</v>
       </c>
     </row>
     <row r="17">
@@ -1123,22 +1123,22 @@
         </is>
       </c>
       <c r="B17" s="21" t="n">
-        <v>1013.4</v>
+        <v>999.5</v>
       </c>
       <c r="C17" s="18" t="n">
-        <v>991.35</v>
+        <v>987.3</v>
       </c>
       <c r="D17" s="7" t="n">
-        <v>993.75</v>
+        <v>994.45</v>
       </c>
       <c r="E17" s="5" t="n">
-        <v>993.6</v>
+        <v>995.85</v>
       </c>
       <c r="F17" s="9" t="n">
         <v>48</v>
       </c>
       <c r="G17" s="5" t="n">
-        <v>1006</v>
+        <v>994.25</v>
       </c>
     </row>
     <row r="18">
@@ -1148,22 +1148,22 @@
         </is>
       </c>
       <c r="B18" s="21" t="n">
-        <v>1906.25</v>
+        <v>1877</v>
       </c>
       <c r="C18" s="18" t="n">
-        <v>1851.65</v>
+        <v>1845</v>
       </c>
       <c r="D18" s="7" t="n">
-        <v>1860.3</v>
+        <v>1856.95</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>1856.65</v>
+        <v>1857.85</v>
       </c>
       <c r="F18" s="9" t="n">
-        <v>84</v>
+        <v>52</v>
       </c>
       <c r="G18" s="5" t="n">
-        <v>1903.5</v>
+        <v>1847.45</v>
       </c>
     </row>
     <row r="19">
@@ -1173,22 +1173,22 @@
         </is>
       </c>
       <c r="B19" s="21" t="n">
-        <v>903.8</v>
+        <v>912.5</v>
       </c>
       <c r="C19" s="18" t="n">
-        <v>890.9</v>
+        <v>892</v>
       </c>
       <c r="D19" s="7" t="n">
-        <v>899</v>
+        <v>907</v>
       </c>
       <c r="E19" s="5" t="n">
-        <v>897</v>
+        <v>906.45</v>
       </c>
       <c r="F19" s="9" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="G19" s="5" t="n">
-        <v>890.9</v>
+        <v>895.25</v>
       </c>
     </row>
     <row r="20">
@@ -1198,22 +1198,22 @@
         </is>
       </c>
       <c r="B20" s="21" t="n">
-        <v>639.65</v>
+        <v>639.95</v>
       </c>
       <c r="C20" s="18" t="n">
-        <v>631.25</v>
+        <v>630.95</v>
       </c>
       <c r="D20" s="7" t="n">
-        <v>636.2</v>
+        <v>637.3</v>
       </c>
       <c r="E20" s="5" t="n">
-        <v>634.7</v>
+        <v>638.8</v>
       </c>
       <c r="F20" s="9" t="n">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="G20" s="5" t="n">
-        <v>631.95</v>
+        <v>636.45</v>
       </c>
     </row>
     <row r="21">
@@ -1223,22 +1223,22 @@
         </is>
       </c>
       <c r="B21" s="21" t="n">
-        <v>2992.8</v>
+        <v>2991.65</v>
       </c>
       <c r="C21" s="18" t="n">
-        <v>2892</v>
+        <v>2921</v>
       </c>
       <c r="D21" s="7" t="n">
-        <v>2904</v>
+        <v>2973.6</v>
       </c>
       <c r="E21" s="5" t="n">
-        <v>2898.7</v>
+        <v>2966.1</v>
       </c>
       <c r="F21" s="9" t="n">
-        <v>44</v>
+        <v>35</v>
       </c>
       <c r="G21" s="5" t="n">
-        <v>2988</v>
+        <v>2925.5</v>
       </c>
     </row>
     <row r="22">
@@ -1248,22 +1248,22 @@
         </is>
       </c>
       <c r="B22" s="21" t="n">
-        <v>276.1</v>
+        <v>274.85</v>
       </c>
       <c r="C22" s="18" t="n">
-        <v>269.85</v>
+        <v>269.35</v>
       </c>
       <c r="D22" s="7" t="n">
-        <v>272.85</v>
+        <v>273.85</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>272</v>
+        <v>273.4</v>
       </c>
       <c r="F22" s="9" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="G22" s="5" t="n">
-        <v>273.55</v>
+        <v>271.1</v>
       </c>
     </row>
     <row r="23">
@@ -1273,22 +1273,22 @@
         </is>
       </c>
       <c r="B23" s="21" t="n">
-        <v>369.65</v>
+        <v>364.75</v>
       </c>
       <c r="C23" s="18" t="n">
-        <v>359.6</v>
+        <v>360.2</v>
       </c>
       <c r="D23" s="7" t="n">
-        <v>365.25</v>
+        <v>363</v>
       </c>
       <c r="E23" s="5" t="n">
-        <v>362.05</v>
+        <v>363.65</v>
       </c>
       <c r="F23" s="9" t="n">
-        <v>168</v>
+        <v>142</v>
       </c>
       <c r="G23" s="5" t="n">
-        <v>367.45</v>
+        <v>362</v>
       </c>
     </row>
     <row r="24">
@@ -1298,22 +1298,22 @@
         </is>
       </c>
       <c r="B24" s="21" t="n">
-        <v>1296.6</v>
+        <v>1299.5</v>
       </c>
       <c r="C24" s="18" t="n">
-        <v>1269.05</v>
+        <v>1275.25</v>
       </c>
       <c r="D24" s="7" t="n">
-        <v>1272.75</v>
+        <v>1291.5</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>1270.8</v>
+        <v>1292.2</v>
       </c>
       <c r="F24" s="9" t="n">
-        <v>150</v>
+        <v>132</v>
       </c>
       <c r="G24" s="5" t="n">
-        <v>1289.65</v>
+        <v>1277.5</v>
       </c>
     </row>
     <row r="25">
@@ -1323,22 +1323,22 @@
         </is>
       </c>
       <c r="B25" s="21" t="n">
-        <v>845.8</v>
+        <v>843.1</v>
       </c>
       <c r="C25" s="18" t="n">
-        <v>835</v>
+        <v>831.55</v>
       </c>
       <c r="D25" s="7" t="n">
-        <v>840.55</v>
+        <v>838.7</v>
       </c>
       <c r="E25" s="5" t="n">
-        <v>838.85</v>
+        <v>838.95</v>
       </c>
       <c r="F25" s="9" t="n">
-        <v>135</v>
+        <v>108</v>
       </c>
       <c r="G25" s="5" t="n">
-        <v>836.45</v>
+        <v>841.8</v>
       </c>
     </row>
     <row r="26">
@@ -1348,22 +1348,22 @@
         </is>
       </c>
       <c r="B26" s="21" t="n">
-        <v>756.95</v>
+        <v>763.45</v>
       </c>
       <c r="C26" s="18" t="n">
-        <v>743</v>
+        <v>746.05</v>
       </c>
       <c r="D26" s="7" t="n">
-        <v>748.05</v>
+        <v>761.8</v>
       </c>
       <c r="E26" s="5" t="n">
-        <v>746.2</v>
+        <v>758.4</v>
       </c>
       <c r="F26" s="9" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G26" s="5" t="n">
-        <v>754.6</v>
+        <v>748.35</v>
       </c>
     </row>
     <row r="27">
@@ -1373,22 +1373,22 @@
         </is>
       </c>
       <c r="B27" s="21" t="n">
-        <v>1120.9</v>
+        <v>1117.5</v>
       </c>
       <c r="C27" s="18" t="n">
-        <v>1095</v>
+        <v>1104.3</v>
       </c>
       <c r="D27" s="7" t="n">
-        <v>1110</v>
+        <v>1110.6</v>
       </c>
       <c r="E27" s="5" t="n">
-        <v>1103.85</v>
+        <v>1111.75</v>
       </c>
       <c r="F27" s="9" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G27" s="5" t="n">
-        <v>1113.95</v>
+        <v>1110.5</v>
       </c>
     </row>
     <row r="28">
@@ -1398,22 +1398,22 @@
         </is>
       </c>
       <c r="B28" s="21" t="n">
-        <v>792.55</v>
+        <v>789.4</v>
       </c>
       <c r="C28" s="18" t="n">
-        <v>778.1</v>
+        <v>777.05</v>
       </c>
       <c r="D28" s="7" t="n">
-        <v>781.5</v>
+        <v>787.35</v>
       </c>
       <c r="E28" s="5" t="n">
-        <v>779.45</v>
+        <v>786.45</v>
       </c>
       <c r="F28" s="9" t="n">
-        <v>109</v>
+        <v>103</v>
       </c>
       <c r="G28" s="5" t="n">
-        <v>785.45</v>
+        <v>778</v>
       </c>
     </row>
     <row r="29">
@@ -1423,22 +1423,22 @@
         </is>
       </c>
       <c r="B29" s="21" t="n">
-        <v>421</v>
+        <v>417.5</v>
       </c>
       <c r="C29" s="18" t="n">
-        <v>412.1</v>
+        <v>410.45</v>
       </c>
       <c r="D29" s="7" t="n">
-        <v>414.8</v>
+        <v>414.45</v>
       </c>
       <c r="E29" s="5" t="n">
-        <v>414.5</v>
+        <v>414.15</v>
       </c>
       <c r="F29" s="23" t="n">
-        <v>98</v>
+        <v>84</v>
       </c>
       <c r="G29" s="24" t="n">
-        <v>417.85</v>
+        <v>413.75</v>
       </c>
     </row>
     <row r="30">
@@ -1448,22 +1448,22 @@
         </is>
       </c>
       <c r="B30" s="22" t="n">
-        <v>145.25</v>
+        <v>145.49</v>
       </c>
       <c r="C30" s="19" t="n">
-        <v>143.09</v>
+        <v>143.1</v>
       </c>
       <c r="D30" s="12" t="n">
-        <v>143.63</v>
+        <v>144.45</v>
       </c>
       <c r="E30" s="15" t="n">
-        <v>143.39</v>
+        <v>144.54</v>
       </c>
       <c r="F30" s="25" t="n">
-        <v>309</v>
+        <v>297</v>
       </c>
       <c r="G30" s="25" t="n">
-        <v>144.89</v>
+        <v>143.29</v>
       </c>
     </row>
     <row r="31" ht="15.75" customHeight="1" thickBot="1">
@@ -1473,22 +1473,22 @@
         </is>
       </c>
       <c r="B31" s="27" t="n">
-        <v>11185</v>
+        <v>11233</v>
       </c>
       <c r="C31" s="26" t="n">
-        <v>10957.6</v>
+        <v>11020</v>
       </c>
       <c r="D31" s="28" t="n">
-        <v>11066</v>
+        <v>11188</v>
       </c>
       <c r="E31" s="10" t="n">
-        <v>10997.8</v>
+        <v>11202.15</v>
       </c>
       <c r="F31" s="29" t="n">
         <v>3</v>
       </c>
       <c r="G31" s="30" t="n">
-        <v>11117.55</v>
+        <v>11047.05</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added exception handling for when csh.xlsx already exists. algo.xlsx too!
</commit_message>
<xml_diff>
--- a/cash high low.xlsx
+++ b/cash high low.xlsx
@@ -748,22 +748,22 @@
         </is>
       </c>
       <c r="B2" s="20" t="n">
-        <v>454.7</v>
+        <v>410.9</v>
       </c>
       <c r="C2" s="17" t="n">
-        <v>445.7</v>
+        <v>403.05</v>
       </c>
       <c r="D2" s="6" t="n">
-        <v>448.8</v>
+        <v>409.5</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>448.4</v>
+        <v>409.5</v>
       </c>
       <c r="F2" s="8" t="n">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>454.5</v>
+        <v>406.75</v>
       </c>
     </row>
     <row r="3">
@@ -773,22 +773,22 @@
         </is>
       </c>
       <c r="B3" s="20" t="n">
-        <v>2526</v>
+        <v>2369.9</v>
       </c>
       <c r="C3" s="17" t="n">
-        <v>2483.15</v>
+        <v>2332.75</v>
       </c>
       <c r="D3" s="6" t="n">
-        <v>2494.8</v>
+        <v>2346</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>2495.85</v>
+        <v>2338.95</v>
       </c>
       <c r="F3" s="8" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="G3" s="4" t="n">
-        <v>2516.25</v>
+        <v>2356.2</v>
       </c>
     </row>
     <row r="4">
@@ -798,22 +798,22 @@
         </is>
       </c>
       <c r="B4" s="21" t="n">
-        <v>557</v>
+        <v>536.3</v>
       </c>
       <c r="C4" s="18" t="n">
-        <v>541.85</v>
+        <v>527</v>
       </c>
       <c r="D4" s="7" t="n">
-        <v>547.35</v>
+        <v>532.15</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>549.1</v>
+        <v>532.1</v>
       </c>
       <c r="F4" s="9" t="n">
-        <v>17</v>
+        <v>6</v>
       </c>
       <c r="G4" s="5" t="n">
-        <v>542.35</v>
+        <v>535.15</v>
       </c>
     </row>
     <row r="5">
@@ -823,22 +823,22 @@
         </is>
       </c>
       <c r="B5" s="21" t="n">
-        <v>1647.55</v>
+        <v>1594.75</v>
       </c>
       <c r="C5" s="18" t="n">
-        <v>1619.2</v>
+        <v>1560.55</v>
       </c>
       <c r="D5" s="7" t="n">
-        <v>1637.1</v>
+        <v>1562.95</v>
       </c>
       <c r="E5" s="5" t="n">
-        <v>1637.05</v>
+        <v>1563.4</v>
       </c>
       <c r="F5" s="9" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="G5" s="5" t="n">
-        <v>1637.1</v>
+        <v>1573.05</v>
       </c>
     </row>
     <row r="6">
@@ -848,22 +848,22 @@
         </is>
       </c>
       <c r="B6" s="21" t="n">
-        <v>6922.1</v>
+        <v>6976.9</v>
       </c>
       <c r="C6" s="18" t="n">
-        <v>6844.8</v>
+        <v>6855.95</v>
       </c>
       <c r="D6" s="7" t="n">
-        <v>6878.95</v>
+        <v>6868</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>6868.35</v>
+        <v>6866.7</v>
       </c>
       <c r="F6" s="9" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="G6" s="5" t="n">
-        <v>6900</v>
+        <v>6952.45</v>
       </c>
     </row>
     <row r="7">
@@ -873,22 +873,22 @@
         </is>
       </c>
       <c r="B7" s="21" t="n">
-        <v>177.03</v>
+        <v>165.41</v>
       </c>
       <c r="C7" s="18" t="n">
-        <v>174.34</v>
+        <v>158.2</v>
       </c>
       <c r="D7" s="7" t="n">
-        <v>174.6</v>
+        <v>164.21</v>
       </c>
       <c r="E7" s="5" t="n">
-        <v>174.55</v>
+        <v>164.38</v>
       </c>
       <c r="F7" s="9" t="n">
-        <v>41</v>
+        <v>135</v>
       </c>
       <c r="G7" s="5" t="n">
-        <v>176.96</v>
+        <v>160.52</v>
       </c>
     </row>
     <row r="8">
@@ -898,22 +898,22 @@
         </is>
       </c>
       <c r="B8" s="21" t="n">
-        <v>264.8</v>
+        <v>247.3</v>
       </c>
       <c r="C8" s="18" t="n">
-        <v>261.32</v>
+        <v>239.05</v>
       </c>
       <c r="D8" s="7" t="n">
-        <v>262.9</v>
+        <v>246.5</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>262.93</v>
+        <v>246.25</v>
       </c>
       <c r="F8" s="9" t="n">
-        <v>97</v>
+        <v>110</v>
       </c>
       <c r="G8" s="5" t="n">
-        <v>262.71</v>
+        <v>241.58</v>
       </c>
     </row>
     <row r="9">
@@ -923,22 +923,22 @@
         </is>
       </c>
       <c r="B9" s="21" t="n">
-        <v>420.25</v>
+        <v>388.6</v>
       </c>
       <c r="C9" s="18" t="n">
-        <v>412.5</v>
+        <v>382.4</v>
       </c>
       <c r="D9" s="7" t="n">
-        <v>414.4</v>
+        <v>383.5</v>
       </c>
       <c r="E9" s="5" t="n">
-        <v>414</v>
+        <v>382.95</v>
       </c>
       <c r="F9" s="9" t="n">
-        <v>66</v>
+        <v>51</v>
       </c>
       <c r="G9" s="5" t="n">
-        <v>420.1</v>
+        <v>385.7</v>
       </c>
     </row>
     <row r="10">
@@ -948,22 +948,22 @@
         </is>
       </c>
       <c r="B10" s="21" t="n">
-        <v>873.4</v>
+        <v>854</v>
       </c>
       <c r="C10" s="18" t="n">
-        <v>858.2</v>
+        <v>837.05</v>
       </c>
       <c r="D10" s="7" t="n">
-        <v>863</v>
+        <v>842.1</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>862.7</v>
+        <v>844.25</v>
       </c>
       <c r="F10" s="9" t="n">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="G10" s="5" t="n">
-        <v>861.4</v>
+        <v>841.85</v>
       </c>
     </row>
     <row r="11">
@@ -973,22 +973,22 @@
         </is>
       </c>
       <c r="B11" s="21" t="n">
-        <v>4873</v>
+        <v>4776.2</v>
       </c>
       <c r="C11" s="18" t="n">
-        <v>4815</v>
+        <v>4698</v>
       </c>
       <c r="D11" s="7" t="n">
-        <v>4857.4</v>
+        <v>4756.95</v>
       </c>
       <c r="E11" s="5" t="n">
-        <v>4842.1</v>
+        <v>4750.55</v>
       </c>
       <c r="F11" s="9" t="n">
         <v>3</v>
       </c>
       <c r="G11" s="5" t="n">
-        <v>4858.05</v>
+        <v>4723.45</v>
       </c>
     </row>
     <row r="12">
@@ -998,22 +998,22 @@
         </is>
       </c>
       <c r="B12" s="21" t="n">
-        <v>215.17</v>
+        <v>197.83</v>
       </c>
       <c r="C12" s="18" t="n">
-        <v>212.31</v>
+        <v>195.05</v>
       </c>
       <c r="D12" s="7" t="n">
-        <v>213.89</v>
+        <v>197</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>213.77</v>
+        <v>197.02</v>
       </c>
       <c r="F12" s="9" t="n">
-        <v>49</v>
+        <v>80</v>
       </c>
       <c r="G12" s="5" t="n">
-        <v>213.9</v>
+        <v>196</v>
       </c>
     </row>
     <row r="13">
@@ -1023,22 +1023,22 @@
         </is>
       </c>
       <c r="B13" s="21" t="n">
-        <v>1925.5</v>
+        <v>1929.65</v>
       </c>
       <c r="C13" s="18" t="n">
-        <v>1901</v>
+        <v>1899.15</v>
       </c>
       <c r="D13" s="7" t="n">
-        <v>1909.95</v>
+        <v>1900.8</v>
       </c>
       <c r="E13" s="5" t="n">
-        <v>1909.9</v>
+        <v>1903</v>
       </c>
       <c r="F13" s="9" t="n">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="G13" s="5" t="n">
-        <v>1925.45</v>
+        <v>1929.45</v>
       </c>
     </row>
     <row r="14">
@@ -1048,22 +1048,22 @@
         </is>
       </c>
       <c r="B14" s="21" t="n">
-        <v>1880</v>
+        <v>1806</v>
       </c>
       <c r="C14" s="18" t="n">
-        <v>1862.05</v>
+        <v>1791.5</v>
       </c>
       <c r="D14" s="7" t="n">
-        <v>1867.55</v>
+        <v>1802</v>
       </c>
       <c r="E14" s="5" t="n">
-        <v>1870</v>
+        <v>1801</v>
       </c>
       <c r="F14" s="9" t="n">
-        <v>134</v>
+        <v>55</v>
       </c>
       <c r="G14" s="5" t="n">
-        <v>1870.1</v>
+        <v>1795.8</v>
       </c>
     </row>
     <row r="15">
@@ -1073,22 +1073,22 @@
         </is>
       </c>
       <c r="B15" s="21" t="n">
-        <v>672.5</v>
+        <v>635.9</v>
       </c>
       <c r="C15" s="18" t="n">
-        <v>654.25</v>
+        <v>628.55</v>
       </c>
       <c r="D15" s="7" t="n">
-        <v>670.3</v>
+        <v>634.3</v>
       </c>
       <c r="E15" s="5" t="n">
-        <v>670.9</v>
+        <v>634.15</v>
       </c>
       <c r="F15" s="9" t="n">
-        <v>50</v>
+        <v>29</v>
       </c>
       <c r="G15" s="5" t="n">
-        <v>668.55</v>
+        <v>633.35</v>
       </c>
     </row>
     <row r="16">
@@ -1098,22 +1098,22 @@
         </is>
       </c>
       <c r="B16" s="21" t="n">
-        <v>1329.05</v>
+        <v>1307</v>
       </c>
       <c r="C16" s="18" t="n">
-        <v>1320.25</v>
+        <v>1287.05</v>
       </c>
       <c r="D16" s="7" t="n">
-        <v>1323.5</v>
+        <v>1297.35</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>1322.3</v>
+        <v>1296.8</v>
       </c>
       <c r="F16" s="9" t="n">
-        <v>80</v>
+        <v>68</v>
       </c>
       <c r="G16" s="5" t="n">
-        <v>1325.4</v>
+        <v>1298.5</v>
       </c>
     </row>
     <row r="17">
@@ -1123,22 +1123,22 @@
         </is>
       </c>
       <c r="B17" s="21" t="n">
-        <v>989.4</v>
+        <v>948.8</v>
       </c>
       <c r="C17" s="18" t="n">
-        <v>977.8</v>
+        <v>930.05</v>
       </c>
       <c r="D17" s="7" t="n">
-        <v>982.75</v>
+        <v>943.5</v>
       </c>
       <c r="E17" s="5" t="n">
-        <v>982.6</v>
+        <v>945.7</v>
       </c>
       <c r="F17" s="9" t="n">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="G17" s="5" t="n">
-        <v>987.75</v>
+        <v>933.9</v>
       </c>
     </row>
     <row r="18">
@@ -1148,22 +1148,22 @@
         </is>
       </c>
       <c r="B18" s="21" t="n">
-        <v>1930.2</v>
+        <v>1937.55</v>
       </c>
       <c r="C18" s="18" t="n">
-        <v>1897.2</v>
+        <v>1909</v>
       </c>
       <c r="D18" s="7" t="n">
-        <v>1926.95</v>
+        <v>1921</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>1923.65</v>
+        <v>1924.3</v>
       </c>
       <c r="F18" s="9" t="n">
-        <v>42</v>
+        <v>27</v>
       </c>
       <c r="G18" s="5" t="n">
-        <v>1908.6</v>
+        <v>1933.25</v>
       </c>
     </row>
     <row r="19">
@@ -1173,22 +1173,22 @@
         </is>
       </c>
       <c r="B19" s="21" t="n">
-        <v>969.6</v>
+        <v>947.5</v>
       </c>
       <c r="C19" s="18" t="n">
-        <v>945.2</v>
+        <v>920.55</v>
       </c>
       <c r="D19" s="7" t="n">
-        <v>968</v>
+        <v>940.05</v>
       </c>
       <c r="E19" s="5" t="n">
-        <v>967.2</v>
+        <v>940.8</v>
       </c>
       <c r="F19" s="9" t="n">
-        <v>14</v>
+        <v>33</v>
       </c>
       <c r="G19" s="5" t="n">
-        <v>953.15</v>
+        <v>925.75</v>
       </c>
     </row>
     <row r="20">
@@ -1198,22 +1198,22 @@
         </is>
       </c>
       <c r="B20" s="21" t="n">
-        <v>638.8</v>
+        <v>587.4</v>
       </c>
       <c r="C20" s="18" t="n">
-        <v>628.95</v>
+        <v>577.1</v>
       </c>
       <c r="D20" s="7" t="n">
-        <v>630.45</v>
+        <v>585.2</v>
       </c>
       <c r="E20" s="5" t="n">
-        <v>630.15</v>
+        <v>583.25</v>
       </c>
       <c r="F20" s="9" t="n">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="G20" s="5" t="n">
-        <v>638.15</v>
+        <v>581.85</v>
       </c>
     </row>
     <row r="21">
@@ -1223,22 +1223,22 @@
         </is>
       </c>
       <c r="B21" s="21" t="n">
-        <v>3071.6</v>
+        <v>2927.55</v>
       </c>
       <c r="C21" s="18" t="n">
-        <v>3040.5</v>
+        <v>2891.1</v>
       </c>
       <c r="D21" s="7" t="n">
-        <v>3048</v>
+        <v>2915</v>
       </c>
       <c r="E21" s="5" t="n">
-        <v>3051.25</v>
+        <v>2909.3</v>
       </c>
       <c r="F21" s="9" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="G21" s="5" t="n">
-        <v>3056</v>
+        <v>2916.2</v>
       </c>
     </row>
     <row r="22">
@@ -1248,22 +1248,22 @@
         </is>
       </c>
       <c r="B22" s="21" t="n">
-        <v>281.25</v>
+        <v>270</v>
       </c>
       <c r="C22" s="18" t="n">
-        <v>278.3</v>
+        <v>264.15</v>
       </c>
       <c r="D22" s="7" t="n">
-        <v>279.5</v>
+        <v>265.15</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>279.15</v>
+        <v>265.15</v>
       </c>
       <c r="F22" s="9" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="G22" s="5" t="n">
-        <v>279.2</v>
+        <v>268.95</v>
       </c>
     </row>
     <row r="23">
@@ -1273,22 +1273,22 @@
         </is>
       </c>
       <c r="B23" s="21" t="n">
-        <v>372.15</v>
+        <v>338.25</v>
       </c>
       <c r="C23" s="18" t="n">
-        <v>367.75</v>
+        <v>330.5</v>
       </c>
       <c r="D23" s="7" t="n">
-        <v>369.45</v>
+        <v>333.3</v>
       </c>
       <c r="E23" s="5" t="n">
-        <v>369.85</v>
+        <v>333.65</v>
       </c>
       <c r="F23" s="9" t="n">
-        <v>108</v>
+        <v>88</v>
       </c>
       <c r="G23" s="5" t="n">
-        <v>370.9</v>
+        <v>332.35</v>
       </c>
     </row>
     <row r="24">
@@ -1298,22 +1298,22 @@
         </is>
       </c>
       <c r="B24" s="21" t="n">
-        <v>1315</v>
+        <v>1227.2</v>
       </c>
       <c r="C24" s="18" t="n">
-        <v>1293.1</v>
+        <v>1213.2</v>
       </c>
       <c r="D24" s="7" t="n">
-        <v>1296.4</v>
+        <v>1223.85</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>1295.15</v>
+        <v>1222.3</v>
       </c>
       <c r="F24" s="9" t="n">
-        <v>146</v>
+        <v>100</v>
       </c>
       <c r="G24" s="5" t="n">
-        <v>1313.6</v>
+        <v>1220.7</v>
       </c>
     </row>
     <row r="25">
@@ -1323,22 +1323,22 @@
         </is>
       </c>
       <c r="B25" s="21" t="n">
-        <v>866.85</v>
+        <v>824</v>
       </c>
       <c r="C25" s="18" t="n">
-        <v>856.95</v>
+        <v>812.2</v>
       </c>
       <c r="D25" s="7" t="n">
-        <v>858.2</v>
+        <v>820.5</v>
       </c>
       <c r="E25" s="5" t="n">
-        <v>858.05</v>
+        <v>821.15</v>
       </c>
       <c r="F25" s="9" t="n">
-        <v>96</v>
+        <v>49</v>
       </c>
       <c r="G25" s="5" t="n">
-        <v>866.85</v>
+        <v>819</v>
       </c>
     </row>
     <row r="26">
@@ -1348,22 +1348,22 @@
         </is>
       </c>
       <c r="B26" s="21" t="n">
-        <v>766.1</v>
+        <v>715.8</v>
       </c>
       <c r="C26" s="18" t="n">
-        <v>752.2</v>
+        <v>695.85</v>
       </c>
       <c r="D26" s="7" t="n">
-        <v>754.95</v>
+        <v>708.95</v>
       </c>
       <c r="E26" s="5" t="n">
-        <v>754.95</v>
+        <v>706.1</v>
       </c>
       <c r="F26" s="9" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G26" s="5" t="n">
-        <v>762.45</v>
+        <v>702.65</v>
       </c>
     </row>
     <row r="27">
@@ -1373,22 +1373,22 @@
         </is>
       </c>
       <c r="B27" s="21" t="n">
-        <v>1119</v>
+        <v>1045</v>
       </c>
       <c r="C27" s="18" t="n">
-        <v>1100.1</v>
+        <v>1025.15</v>
       </c>
       <c r="D27" s="7" t="n">
-        <v>1109</v>
+        <v>1035</v>
       </c>
       <c r="E27" s="5" t="n">
-        <v>1106.05</v>
+        <v>1034.25</v>
       </c>
       <c r="F27" s="9" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G27" s="5" t="n">
-        <v>1119</v>
+        <v>1031.45</v>
       </c>
     </row>
     <row r="28">
@@ -1398,22 +1398,22 @@
         </is>
       </c>
       <c r="B28" s="21" t="n">
-        <v>819.2</v>
+        <v>733.7</v>
       </c>
       <c r="C28" s="18" t="n">
-        <v>797</v>
+        <v>717.7</v>
       </c>
       <c r="D28" s="7" t="n">
-        <v>799.7</v>
+        <v>721.5</v>
       </c>
       <c r="E28" s="5" t="n">
-        <v>798.75</v>
+        <v>722.2</v>
       </c>
       <c r="F28" s="9" t="n">
-        <v>155</v>
+        <v>96</v>
       </c>
       <c r="G28" s="5" t="n">
-        <v>818.75</v>
+        <v>728.55</v>
       </c>
     </row>
     <row r="29">
@@ -1423,22 +1423,22 @@
         </is>
       </c>
       <c r="B29" s="21" t="n">
-        <v>447.7</v>
+        <v>405</v>
       </c>
       <c r="C29" s="18" t="n">
-        <v>439.1</v>
+        <v>396.85</v>
       </c>
       <c r="D29" s="7" t="n">
-        <v>440.65</v>
+        <v>399.7</v>
       </c>
       <c r="E29" s="5" t="n">
-        <v>440.75</v>
+        <v>399.9</v>
       </c>
       <c r="F29" s="23" t="n">
-        <v>134</v>
+        <v>90</v>
       </c>
       <c r="G29" s="24" t="n">
-        <v>446.45</v>
+        <v>403.55</v>
       </c>
     </row>
     <row r="30">
@@ -1448,22 +1448,22 @@
         </is>
       </c>
       <c r="B30" s="22" t="n">
-        <v>150.67</v>
+        <v>143.75</v>
       </c>
       <c r="C30" s="19" t="n">
-        <v>146.63</v>
+        <v>140.61</v>
       </c>
       <c r="D30" s="12" t="n">
-        <v>149.7</v>
+        <v>141.81</v>
       </c>
       <c r="E30" s="15" t="n">
-        <v>149.88</v>
+        <v>141.71</v>
       </c>
       <c r="F30" s="25" t="n">
-        <v>390</v>
+        <v>275</v>
       </c>
       <c r="G30" s="25" t="n">
-        <v>147.9</v>
+        <v>142.78</v>
       </c>
     </row>
     <row r="31" ht="15.75" customHeight="1" thickBot="1">
@@ -1473,22 +1473,22 @@
         </is>
       </c>
       <c r="B31" s="27" t="n">
-        <v>11861</v>
+        <v>11539.35</v>
       </c>
       <c r="C31" s="26" t="n">
-        <v>11718</v>
+        <v>11375</v>
       </c>
       <c r="D31" s="28" t="n">
-        <v>11795.2</v>
+        <v>11465</v>
       </c>
       <c r="E31" s="10" t="n">
-        <v>11814.8</v>
+        <v>11472.6</v>
       </c>
       <c r="F31" s="29" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G31" s="30" t="n">
-        <v>11770.75</v>
+        <v>11470</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added colaind and changed LTP to be taken from NSE site instead of csh.xlsx or algo.xlsx
</commit_message>
<xml_diff>
--- a/cash high low.xlsx
+++ b/cash high low.xlsx
@@ -367,7 +367,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="2" pivotButton="0" quotePrefix="0" xfId="1"/>
@@ -399,13 +399,85 @@
     <xf numFmtId="2" fontId="2" fillId="2" borderId="22" pivotButton="0" quotePrefix="0" xfId="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="21" pivotButton="0" quotePrefix="0" xfId="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="21" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="2" fillId="2" borderId="4" pivotButton="0" quotePrefix="0" xfId="1"/>
+    <xf numFmtId="2" fontId="2" fillId="2" borderId="5" pivotButton="0" quotePrefix="0" xfId="1"/>
+    <xf numFmtId="2" fontId="2" fillId="2" borderId="15" pivotButton="0" quotePrefix="0" xfId="1"/>
+    <xf numFmtId="2" fontId="2" fillId="2" borderId="8" pivotButton="0" quotePrefix="0" xfId="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Calculation" xfId="1" builtinId="22"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleMedium9"/>
-  <colors/>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -748,22 +820,22 @@
         </is>
       </c>
       <c r="B2" s="20" t="n">
-        <v>410.9</v>
+        <v>444.4</v>
       </c>
       <c r="C2" s="17" t="n">
-        <v>403.05</v>
+        <v>435.9</v>
       </c>
       <c r="D2" s="6" t="n">
-        <v>409.5</v>
-      </c>
-      <c r="E2" s="4" t="n">
-        <v>409.5</v>
+        <v>442.8</v>
+      </c>
+      <c r="E2" s="32" t="n">
+        <v>442.7</v>
       </c>
       <c r="F2" s="8" t="n">
         <v>13</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>406.75</v>
+        <v>436.9</v>
       </c>
     </row>
     <row r="3">
@@ -773,22 +845,22 @@
         </is>
       </c>
       <c r="B3" s="20" t="n">
-        <v>2369.9</v>
+        <v>2424.5</v>
       </c>
       <c r="C3" s="17" t="n">
-        <v>2332.75</v>
+        <v>2380.05</v>
       </c>
       <c r="D3" s="6" t="n">
-        <v>2346</v>
-      </c>
-      <c r="E3" s="4" t="n">
-        <v>2338.95</v>
+        <v>2399.5</v>
+      </c>
+      <c r="E3" s="32" t="n">
+        <v>2399.8</v>
       </c>
       <c r="F3" s="8" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="G3" s="4" t="n">
-        <v>2356.2</v>
+        <v>2410.4</v>
       </c>
     </row>
     <row r="4">
@@ -798,22 +870,22 @@
         </is>
       </c>
       <c r="B4" s="21" t="n">
-        <v>536.3</v>
+        <v>455.75</v>
       </c>
       <c r="C4" s="18" t="n">
-        <v>527</v>
+        <v>449</v>
       </c>
       <c r="D4" s="7" t="n">
-        <v>532.15</v>
-      </c>
-      <c r="E4" s="5" t="n">
-        <v>532.1</v>
+        <v>452.7</v>
+      </c>
+      <c r="E4" s="33" t="n">
+        <v>452.8</v>
       </c>
       <c r="F4" s="9" t="n">
         <v>6</v>
       </c>
       <c r="G4" s="5" t="n">
-        <v>535.15</v>
+        <v>452.8</v>
       </c>
     </row>
     <row r="5">
@@ -823,22 +895,22 @@
         </is>
       </c>
       <c r="B5" s="21" t="n">
-        <v>1594.75</v>
+        <v>1698.4</v>
       </c>
       <c r="C5" s="18" t="n">
-        <v>1560.55</v>
+        <v>1674.35</v>
       </c>
       <c r="D5" s="7" t="n">
-        <v>1562.95</v>
-      </c>
-      <c r="E5" s="5" t="n">
-        <v>1563.4</v>
+        <v>1682.7</v>
+      </c>
+      <c r="E5" s="33" t="n">
+        <v>1680.65</v>
       </c>
       <c r="F5" s="9" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="G5" s="5" t="n">
-        <v>1573.05</v>
+        <v>1677</v>
       </c>
     </row>
     <row r="6">
@@ -848,22 +920,22 @@
         </is>
       </c>
       <c r="B6" s="21" t="n">
-        <v>6976.9</v>
+        <v>7284.95</v>
       </c>
       <c r="C6" s="18" t="n">
-        <v>6855.95</v>
+        <v>7173.15</v>
       </c>
       <c r="D6" s="7" t="n">
-        <v>6868</v>
-      </c>
-      <c r="E6" s="5" t="n">
-        <v>6866.7</v>
+        <v>7185</v>
+      </c>
+      <c r="E6" s="33" t="n">
+        <v>7182.1</v>
       </c>
       <c r="F6" s="9" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G6" s="5" t="n">
-        <v>6952.45</v>
+        <v>7194.25</v>
       </c>
     </row>
     <row r="7">
@@ -873,22 +945,22 @@
         </is>
       </c>
       <c r="B7" s="21" t="n">
-        <v>165.41</v>
+        <v>151.94</v>
       </c>
       <c r="C7" s="18" t="n">
-        <v>158.2</v>
+        <v>149.52</v>
       </c>
       <c r="D7" s="7" t="n">
-        <v>164.21</v>
-      </c>
-      <c r="E7" s="5" t="n">
-        <v>164.38</v>
+        <v>151.3</v>
+      </c>
+      <c r="E7" s="33" t="n">
+        <v>151.24</v>
       </c>
       <c r="F7" s="9" t="n">
-        <v>135</v>
+        <v>35</v>
       </c>
       <c r="G7" s="5" t="n">
-        <v>160.52</v>
+        <v>149.63</v>
       </c>
     </row>
     <row r="8">
@@ -898,22 +970,22 @@
         </is>
       </c>
       <c r="B8" s="21" t="n">
-        <v>247.3</v>
+        <v>228.9</v>
       </c>
       <c r="C8" s="18" t="n">
-        <v>239.05</v>
+        <v>225.84</v>
       </c>
       <c r="D8" s="7" t="n">
-        <v>246.5</v>
-      </c>
-      <c r="E8" s="5" t="n">
-        <v>246.25</v>
+        <v>227.9</v>
+      </c>
+      <c r="E8" s="33" t="n">
+        <v>228</v>
       </c>
       <c r="F8" s="9" t="n">
-        <v>110</v>
+        <v>60</v>
       </c>
       <c r="G8" s="5" t="n">
-        <v>241.58</v>
+        <v>228.26</v>
       </c>
     </row>
     <row r="9">
@@ -923,22 +995,22 @@
         </is>
       </c>
       <c r="B9" s="21" t="n">
-        <v>388.6</v>
+        <v>389.3</v>
       </c>
       <c r="C9" s="18" t="n">
-        <v>382.4</v>
+        <v>382.05</v>
       </c>
       <c r="D9" s="7" t="n">
-        <v>383.5</v>
-      </c>
-      <c r="E9" s="5" t="n">
-        <v>382.95</v>
+        <v>388.4</v>
+      </c>
+      <c r="E9" s="33" t="n">
+        <v>387.65</v>
       </c>
       <c r="F9" s="9" t="n">
-        <v>51</v>
+        <v>83</v>
       </c>
       <c r="G9" s="5" t="n">
-        <v>385.7</v>
+        <v>382.55</v>
       </c>
     </row>
     <row r="10">
@@ -948,22 +1020,22 @@
         </is>
       </c>
       <c r="B10" s="21" t="n">
-        <v>854</v>
+        <v>753.55</v>
       </c>
       <c r="C10" s="18" t="n">
-        <v>837.05</v>
+        <v>742.5</v>
       </c>
       <c r="D10" s="7" t="n">
-        <v>842.1</v>
-      </c>
-      <c r="E10" s="5" t="n">
-        <v>844.25</v>
+        <v>750</v>
+      </c>
+      <c r="E10" s="33" t="n">
+        <v>749</v>
       </c>
       <c r="F10" s="9" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="G10" s="5" t="n">
-        <v>841.85</v>
+        <v>743.5</v>
       </c>
     </row>
     <row r="11">
@@ -973,22 +1045,22 @@
         </is>
       </c>
       <c r="B11" s="21" t="n">
-        <v>4776.2</v>
+        <v>5075.4</v>
       </c>
       <c r="C11" s="18" t="n">
-        <v>4698</v>
+        <v>4998.05</v>
       </c>
       <c r="D11" s="7" t="n">
-        <v>4756.95</v>
-      </c>
-      <c r="E11" s="5" t="n">
-        <v>4750.55</v>
+        <v>5021.25</v>
+      </c>
+      <c r="E11" s="33" t="n">
+        <v>5012.3</v>
       </c>
       <c r="F11" s="9" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G11" s="5" t="n">
-        <v>4723.45</v>
+        <v>5022</v>
       </c>
     </row>
     <row r="12">
@@ -998,22 +1070,22 @@
         </is>
       </c>
       <c r="B12" s="21" t="n">
-        <v>197.83</v>
+        <v>194.53</v>
       </c>
       <c r="C12" s="18" t="n">
-        <v>195.05</v>
+        <v>191.27</v>
       </c>
       <c r="D12" s="7" t="n">
-        <v>197</v>
-      </c>
-      <c r="E12" s="5" t="n">
-        <v>197.02</v>
+        <v>191.7</v>
+      </c>
+      <c r="E12" s="33" t="n">
+        <v>191.58</v>
       </c>
       <c r="F12" s="9" t="n">
         <v>80</v>
       </c>
       <c r="G12" s="5" t="n">
-        <v>196</v>
+        <v>194.35</v>
       </c>
     </row>
     <row r="13">
@@ -1023,22 +1095,22 @@
         </is>
       </c>
       <c r="B13" s="21" t="n">
-        <v>1929.65</v>
+        <v>1793.1</v>
       </c>
       <c r="C13" s="18" t="n">
-        <v>1899.15</v>
+        <v>1750.05</v>
       </c>
       <c r="D13" s="7" t="n">
-        <v>1900.8</v>
-      </c>
-      <c r="E13" s="5" t="n">
-        <v>1903</v>
+        <v>1789.45</v>
+      </c>
+      <c r="E13" s="33" t="n">
+        <v>1788.9</v>
       </c>
       <c r="F13" s="9" t="n">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="G13" s="5" t="n">
-        <v>1929.45</v>
+        <v>1751.15</v>
       </c>
     </row>
     <row r="14">
@@ -1048,22 +1120,22 @@
         </is>
       </c>
       <c r="B14" s="21" t="n">
-        <v>1806</v>
+        <v>1645.85</v>
       </c>
       <c r="C14" s="18" t="n">
-        <v>1791.5</v>
+        <v>1628.5</v>
       </c>
       <c r="D14" s="7" t="n">
-        <v>1802</v>
-      </c>
-      <c r="E14" s="5" t="n">
-        <v>1801</v>
+        <v>1636.7</v>
+      </c>
+      <c r="E14" s="33" t="n">
+        <v>1636.75</v>
       </c>
       <c r="F14" s="9" t="n">
-        <v>55</v>
+        <v>115</v>
       </c>
       <c r="G14" s="5" t="n">
-        <v>1795.8</v>
+        <v>1645.3</v>
       </c>
     </row>
     <row r="15">
@@ -1073,22 +1145,22 @@
         </is>
       </c>
       <c r="B15" s="21" t="n">
-        <v>635.9</v>
+        <v>619</v>
       </c>
       <c r="C15" s="18" t="n">
-        <v>628.55</v>
+        <v>610</v>
       </c>
       <c r="D15" s="7" t="n">
-        <v>634.3</v>
-      </c>
-      <c r="E15" s="5" t="n">
-        <v>634.15</v>
+        <v>616</v>
+      </c>
+      <c r="E15" s="33" t="n">
+        <v>617</v>
       </c>
       <c r="F15" s="9" t="n">
-        <v>29</v>
+        <v>64</v>
       </c>
       <c r="G15" s="5" t="n">
-        <v>633.35</v>
+        <v>610.95</v>
       </c>
     </row>
     <row r="16">
@@ -1098,22 +1170,22 @@
         </is>
       </c>
       <c r="B16" s="21" t="n">
-        <v>1307</v>
+        <v>1240.95</v>
       </c>
       <c r="C16" s="18" t="n">
-        <v>1287.05</v>
+        <v>1218</v>
       </c>
       <c r="D16" s="7" t="n">
-        <v>1297.35</v>
-      </c>
-      <c r="E16" s="5" t="n">
-        <v>1296.8</v>
+        <v>1225.15</v>
+      </c>
+      <c r="E16" s="33" t="n">
+        <v>1225.45</v>
       </c>
       <c r="F16" s="9" t="n">
-        <v>68</v>
+        <v>97</v>
       </c>
       <c r="G16" s="5" t="n">
-        <v>1298.5</v>
+        <v>1239.45</v>
       </c>
     </row>
     <row r="17">
@@ -1123,22 +1195,22 @@
         </is>
       </c>
       <c r="B17" s="21" t="n">
-        <v>948.8</v>
+        <v>975.6</v>
       </c>
       <c r="C17" s="18" t="n">
-        <v>930.05</v>
+        <v>959</v>
       </c>
       <c r="D17" s="7" t="n">
-        <v>943.5</v>
-      </c>
-      <c r="E17" s="5" t="n">
-        <v>945.7</v>
+        <v>972.9</v>
+      </c>
+      <c r="E17" s="33" t="n">
+        <v>970.95</v>
       </c>
       <c r="F17" s="9" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="G17" s="5" t="n">
-        <v>933.9</v>
+        <v>961.5</v>
       </c>
     </row>
     <row r="18">
@@ -1148,22 +1220,22 @@
         </is>
       </c>
       <c r="B18" s="21" t="n">
-        <v>1937.55</v>
+        <v>1851.1</v>
       </c>
       <c r="C18" s="18" t="n">
-        <v>1909</v>
+        <v>1812</v>
       </c>
       <c r="D18" s="7" t="n">
-        <v>1921</v>
-      </c>
-      <c r="E18" s="5" t="n">
-        <v>1924.3</v>
+        <v>1817.5</v>
+      </c>
+      <c r="E18" s="33" t="n">
+        <v>1815.45</v>
       </c>
       <c r="F18" s="9" t="n">
-        <v>27</v>
+        <v>164</v>
       </c>
       <c r="G18" s="5" t="n">
-        <v>1933.25</v>
+        <v>1844.55</v>
       </c>
     </row>
     <row r="19">
@@ -1173,22 +1245,22 @@
         </is>
       </c>
       <c r="B19" s="21" t="n">
-        <v>947.5</v>
+        <v>930.9</v>
       </c>
       <c r="C19" s="18" t="n">
-        <v>920.55</v>
+        <v>916.5</v>
       </c>
       <c r="D19" s="7" t="n">
-        <v>940.05</v>
-      </c>
-      <c r="E19" s="5" t="n">
-        <v>940.8</v>
+        <v>924.9</v>
+      </c>
+      <c r="E19" s="33" t="n">
+        <v>924.65</v>
       </c>
       <c r="F19" s="9" t="n">
-        <v>33</v>
+        <v>13</v>
       </c>
       <c r="G19" s="5" t="n">
-        <v>925.75</v>
+        <v>918</v>
       </c>
     </row>
     <row r="20">
@@ -1198,22 +1270,22 @@
         </is>
       </c>
       <c r="B20" s="21" t="n">
-        <v>587.4</v>
+        <v>566.95</v>
       </c>
       <c r="C20" s="18" t="n">
-        <v>577.1</v>
+        <v>557.25</v>
       </c>
       <c r="D20" s="7" t="n">
-        <v>585.2</v>
-      </c>
-      <c r="E20" s="5" t="n">
-        <v>583.25</v>
+        <v>562.95</v>
+      </c>
+      <c r="E20" s="33" t="n">
+        <v>562.7</v>
       </c>
       <c r="F20" s="9" t="n">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="G20" s="5" t="n">
-        <v>581.85</v>
+        <v>562.6</v>
       </c>
     </row>
     <row r="21">
@@ -1223,22 +1295,22 @@
         </is>
       </c>
       <c r="B21" s="21" t="n">
-        <v>2927.55</v>
+        <v>2968.3</v>
       </c>
       <c r="C21" s="18" t="n">
-        <v>2891.1</v>
+        <v>2903.1</v>
       </c>
       <c r="D21" s="7" t="n">
-        <v>2915</v>
-      </c>
-      <c r="E21" s="5" t="n">
-        <v>2909.3</v>
+        <v>2922.35</v>
+      </c>
+      <c r="E21" s="33" t="n">
+        <v>2917.35</v>
       </c>
       <c r="F21" s="9" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G21" s="5" t="n">
-        <v>2916.2</v>
+        <v>2933.45</v>
       </c>
     </row>
     <row r="22">
@@ -1248,22 +1320,22 @@
         </is>
       </c>
       <c r="B22" s="21" t="n">
-        <v>270</v>
+        <v>274.5</v>
       </c>
       <c r="C22" s="18" t="n">
-        <v>264.15</v>
+        <v>267.75</v>
       </c>
       <c r="D22" s="7" t="n">
-        <v>265.15</v>
-      </c>
-      <c r="E22" s="5" t="n">
-        <v>265.15</v>
+        <v>268</v>
+      </c>
+      <c r="E22" s="33" t="n">
+        <v>268.55</v>
       </c>
       <c r="F22" s="9" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="G22" s="5" t="n">
-        <v>268.95</v>
+        <v>268.8</v>
       </c>
     </row>
     <row r="23">
@@ -1273,22 +1345,22 @@
         </is>
       </c>
       <c r="B23" s="21" t="n">
-        <v>338.25</v>
+        <v>329</v>
       </c>
       <c r="C23" s="18" t="n">
-        <v>330.5</v>
+        <v>325</v>
       </c>
       <c r="D23" s="7" t="n">
-        <v>333.3</v>
-      </c>
-      <c r="E23" s="5" t="n">
-        <v>333.65</v>
+        <v>326</v>
+      </c>
+      <c r="E23" s="33" t="n">
+        <v>326.15</v>
       </c>
       <c r="F23" s="9" t="n">
-        <v>88</v>
+        <v>71</v>
       </c>
       <c r="G23" s="5" t="n">
-        <v>332.35</v>
+        <v>325.65</v>
       </c>
     </row>
     <row r="24">
@@ -1298,22 +1370,22 @@
         </is>
       </c>
       <c r="B24" s="21" t="n">
-        <v>1227.2</v>
+        <v>1306.4</v>
       </c>
       <c r="C24" s="18" t="n">
-        <v>1213.2</v>
+        <v>1285</v>
       </c>
       <c r="D24" s="7" t="n">
-        <v>1223.85</v>
-      </c>
-      <c r="E24" s="5" t="n">
-        <v>1222.3</v>
+        <v>1300</v>
+      </c>
+      <c r="E24" s="33" t="n">
+        <v>1302.35</v>
       </c>
       <c r="F24" s="9" t="n">
-        <v>100</v>
+        <v>293</v>
       </c>
       <c r="G24" s="5" t="n">
-        <v>1220.7</v>
+        <v>1302.3</v>
       </c>
     </row>
     <row r="25">
@@ -1323,22 +1395,22 @@
         </is>
       </c>
       <c r="B25" s="21" t="n">
-        <v>824</v>
+        <v>767.95</v>
       </c>
       <c r="C25" s="18" t="n">
-        <v>812.2</v>
+        <v>759.4</v>
       </c>
       <c r="D25" s="7" t="n">
-        <v>820.5</v>
-      </c>
-      <c r="E25" s="5" t="n">
-        <v>821.15</v>
+        <v>763.8</v>
+      </c>
+      <c r="E25" s="33" t="n">
+        <v>764.1</v>
       </c>
       <c r="F25" s="9" t="n">
-        <v>49</v>
+        <v>57</v>
       </c>
       <c r="G25" s="5" t="n">
-        <v>819</v>
+        <v>764.7</v>
       </c>
     </row>
     <row r="26">
@@ -1348,22 +1420,22 @@
         </is>
       </c>
       <c r="B26" s="21" t="n">
-        <v>715.8</v>
+        <v>658.5</v>
       </c>
       <c r="C26" s="18" t="n">
-        <v>695.85</v>
+        <v>648</v>
       </c>
       <c r="D26" s="7" t="n">
-        <v>708.95</v>
-      </c>
-      <c r="E26" s="5" t="n">
-        <v>706.1</v>
+        <v>653.4</v>
+      </c>
+      <c r="E26" s="33" t="n">
+        <v>649.35</v>
       </c>
       <c r="F26" s="9" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G26" s="5" t="n">
-        <v>702.65</v>
+        <v>654</v>
       </c>
     </row>
     <row r="27">
@@ -1373,22 +1445,22 @@
         </is>
       </c>
       <c r="B27" s="21" t="n">
-        <v>1045</v>
+        <v>986.95</v>
       </c>
       <c r="C27" s="18" t="n">
-        <v>1025.15</v>
+        <v>968.75</v>
       </c>
       <c r="D27" s="7" t="n">
-        <v>1035</v>
-      </c>
-      <c r="E27" s="5" t="n">
-        <v>1034.25</v>
+        <v>974</v>
+      </c>
+      <c r="E27" s="33" t="n">
+        <v>975.35</v>
       </c>
       <c r="F27" s="9" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="G27" s="5" t="n">
-        <v>1031.45</v>
+        <v>984.7</v>
       </c>
     </row>
     <row r="28">
@@ -1398,22 +1470,22 @@
         </is>
       </c>
       <c r="B28" s="21" t="n">
-        <v>733.7</v>
+        <v>785.5</v>
       </c>
       <c r="C28" s="18" t="n">
-        <v>717.7</v>
+        <v>774.6</v>
       </c>
       <c r="D28" s="7" t="n">
-        <v>721.5</v>
-      </c>
-      <c r="E28" s="5" t="n">
-        <v>722.2</v>
+        <v>779.9</v>
+      </c>
+      <c r="E28" s="33" t="n">
+        <v>779.75</v>
       </c>
       <c r="F28" s="9" t="n">
-        <v>96</v>
+        <v>70</v>
       </c>
       <c r="G28" s="5" t="n">
-        <v>728.55</v>
+        <v>776.55</v>
       </c>
     </row>
     <row r="29">
@@ -1423,22 +1495,22 @@
         </is>
       </c>
       <c r="B29" s="21" t="n">
-        <v>405</v>
+        <v>375.4</v>
       </c>
       <c r="C29" s="18" t="n">
-        <v>396.85</v>
+        <v>366.4</v>
       </c>
       <c r="D29" s="7" t="n">
-        <v>399.7</v>
-      </c>
-      <c r="E29" s="5" t="n">
-        <v>399.9</v>
+        <v>373.5</v>
+      </c>
+      <c r="E29" s="33" t="n">
+        <v>373.6</v>
       </c>
       <c r="F29" s="23" t="n">
-        <v>90</v>
+        <v>55</v>
       </c>
       <c r="G29" s="24" t="n">
-        <v>403.55</v>
+        <v>367.3</v>
       </c>
     </row>
     <row r="30">
@@ -1448,22 +1520,22 @@
         </is>
       </c>
       <c r="B30" s="22" t="n">
-        <v>143.75</v>
+        <v>131.16</v>
       </c>
       <c r="C30" s="19" t="n">
-        <v>140.61</v>
+        <v>127.66</v>
       </c>
       <c r="D30" s="12" t="n">
-        <v>141.81</v>
-      </c>
-      <c r="E30" s="15" t="n">
-        <v>141.71</v>
+        <v>130.15</v>
+      </c>
+      <c r="E30" s="34" t="n">
+        <v>130.28</v>
       </c>
       <c r="F30" s="25" t="n">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="G30" s="25" t="n">
-        <v>142.78</v>
+        <v>127.94</v>
       </c>
     </row>
     <row r="31" ht="15.75" customHeight="1" thickBot="1">
@@ -1473,22 +1545,22 @@
         </is>
       </c>
       <c r="B31" s="27" t="n">
-        <v>11539.35</v>
+        <v>10723.95</v>
       </c>
       <c r="C31" s="26" t="n">
-        <v>11375</v>
+        <v>10500.1</v>
       </c>
       <c r="D31" s="28" t="n">
-        <v>11465</v>
-      </c>
-      <c r="E31" s="10" t="n">
-        <v>11472.6</v>
+        <v>10600</v>
+      </c>
+      <c r="E31" s="35" t="n">
+        <v>10580</v>
       </c>
       <c r="F31" s="29" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G31" s="30" t="n">
-        <v>11470</v>
+        <v>10639.7</v>
       </c>
     </row>
   </sheetData>
@@ -1505,6 +1577,9 @@
   </sheetPr>
   <dimension ref="A1:O38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10.42578125" bestFit="1" customWidth="1" min="10" max="10"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="n"/>
@@ -1629,6 +1704,9 @@
       <c r="E8" s="1" t="n"/>
       <c r="F8" s="1" t="n"/>
       <c r="G8" s="1" t="n"/>
+      <c r="J8" s="31" t="n">
+        <v>45309</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
@@ -1643,22 +1721,22 @@
       <c r="F9" s="1" t="n"/>
       <c r="G9" s="1" t="n"/>
       <c r="J9" t="n">
-        <v>587.5</v>
+        <v>444.4</v>
       </c>
       <c r="K9" t="n">
-        <v>579.1</v>
+        <v>435.9</v>
       </c>
       <c r="L9" t="n">
-        <v>582.15</v>
+        <v>442.8</v>
       </c>
       <c r="M9" t="n">
-        <v>582.95</v>
+        <v>442.8</v>
       </c>
       <c r="N9" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="O9" t="n">
-        <v>586</v>
+        <v>436.9</v>
       </c>
     </row>
     <row r="10">
@@ -1674,22 +1752,22 @@
       <c r="F10" s="1" t="n"/>
       <c r="G10" s="1" t="n"/>
       <c r="J10" t="n">
-        <v>3179</v>
+        <v>2424.5</v>
       </c>
       <c r="K10" t="n">
-        <v>3116</v>
+        <v>2380.05</v>
       </c>
       <c r="L10" t="n">
-        <v>3131</v>
+        <v>2399.5</v>
       </c>
       <c r="M10" t="n">
-        <v>3135.85</v>
+        <v>2399.8</v>
       </c>
       <c r="N10" t="n">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="O10" t="n">
-        <v>3127</v>
+        <v>2410.4</v>
       </c>
     </row>
     <row r="11">
@@ -1705,22 +1783,22 @@
       <c r="F11" s="1" t="n"/>
       <c r="G11" s="1" t="n"/>
       <c r="J11" t="n">
-        <v>555.9</v>
+        <v>455.75</v>
       </c>
       <c r="K11" t="n">
-        <v>545</v>
+        <v>449</v>
       </c>
       <c r="L11" t="n">
-        <v>547.9</v>
+        <v>452.7</v>
       </c>
       <c r="M11" t="n">
-        <v>547.85</v>
+        <v>452.8</v>
       </c>
       <c r="N11" t="n">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="O11" t="n">
-        <v>551.25</v>
+        <v>452.8</v>
       </c>
     </row>
     <row r="12">
@@ -1736,22 +1814,22 @@
       <c r="F12" s="1" t="n"/>
       <c r="G12" s="1" t="n"/>
       <c r="J12" t="n">
-        <v>2029.9</v>
+        <v>1698.4</v>
       </c>
       <c r="K12" t="n">
-        <v>1971.2</v>
+        <v>1674.35</v>
       </c>
       <c r="L12" t="n">
-        <v>1969.65</v>
+        <v>1682.7</v>
       </c>
       <c r="M12" t="n">
-        <v>1973.4</v>
+        <v>1682.7</v>
       </c>
       <c r="N12" t="n">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="O12" t="n">
-        <v>1973</v>
+        <v>1677</v>
       </c>
     </row>
     <row r="13">
@@ -1767,22 +1845,22 @@
       <c r="F13" s="1" t="n"/>
       <c r="G13" s="1" t="n"/>
       <c r="J13" t="n">
-        <v>7810</v>
+        <v>7284.95</v>
       </c>
       <c r="K13" t="n">
-        <v>7712</v>
+        <v>7173.15</v>
       </c>
       <c r="L13" t="n">
-        <v>7697.85</v>
+        <v>7185</v>
       </c>
       <c r="M13" t="n">
-        <v>7703</v>
+        <v>7182</v>
       </c>
       <c r="N13" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="O13" t="n">
-        <v>7714.5</v>
+        <v>7194.25</v>
       </c>
     </row>
     <row r="14">
@@ -1798,22 +1876,22 @@
       <c r="F14" s="1" t="n"/>
       <c r="G14" s="1" t="n"/>
       <c r="J14" t="n">
-        <v>3209.9</v>
+        <v>151.94</v>
       </c>
       <c r="K14" t="n">
-        <v>3120.6</v>
+        <v>149.52</v>
       </c>
       <c r="L14" t="n">
-        <v>198.45</v>
+        <v>151.3</v>
       </c>
       <c r="M14" t="n">
-        <v>198.74</v>
+        <v>151.24</v>
       </c>
       <c r="N14" t="n">
-        <v>94</v>
+        <v>35</v>
       </c>
       <c r="O14" t="n">
-        <v>3143</v>
+        <v>149.63</v>
       </c>
     </row>
     <row r="15">
@@ -1829,22 +1907,22 @@
       <c r="F15" s="1" t="n"/>
       <c r="G15" s="1" t="n"/>
       <c r="J15" t="n">
-        <v>551</v>
+        <v>228.9</v>
       </c>
       <c r="K15" t="n">
-        <v>538.5</v>
+        <v>225.84</v>
       </c>
       <c r="L15" t="n">
-        <v>247</v>
+        <v>227.9</v>
       </c>
       <c r="M15" t="n">
-        <v>247.8</v>
+        <v>228</v>
       </c>
       <c r="N15" t="n">
-        <v>129</v>
+        <v>60</v>
       </c>
       <c r="O15" t="n">
-        <v>543.8</v>
+        <v>228.26</v>
       </c>
     </row>
     <row r="16">
@@ -1860,22 +1938,22 @@
       <c r="F16" s="1" t="n"/>
       <c r="G16" s="1" t="n"/>
       <c r="J16" t="n">
-        <v>2018.95</v>
+        <v>389.3</v>
       </c>
       <c r="K16" t="n">
-        <v>1968.3</v>
+        <v>382.05</v>
       </c>
       <c r="L16" t="n">
-        <v>509.4</v>
+        <v>388.4</v>
       </c>
       <c r="M16" t="n">
-        <v>510.15</v>
+        <v>387.65</v>
       </c>
       <c r="N16" t="n">
-        <v>88</v>
+        <v>83</v>
       </c>
       <c r="O16" t="n">
-        <v>2008.3</v>
+        <v>382.55</v>
       </c>
     </row>
     <row r="17">
@@ -1891,22 +1969,22 @@
       <c r="F17" s="1" t="n"/>
       <c r="G17" s="1" t="n"/>
       <c r="J17" t="n">
-        <v>7800</v>
+        <v>753.55</v>
       </c>
       <c r="K17" t="n">
-        <v>7676.15</v>
+        <v>742.5</v>
       </c>
       <c r="L17" t="n">
-        <v>895.45</v>
+        <v>750</v>
       </c>
       <c r="M17" t="n">
-        <v>895.15</v>
+        <v>749</v>
       </c>
       <c r="N17" t="n">
-        <v>46</v>
+        <v>20</v>
       </c>
       <c r="O17" t="n">
-        <v>7757.75</v>
+        <v>743.5</v>
       </c>
     </row>
     <row r="18">
@@ -1922,22 +2000,22 @@
       <c r="F18" s="1" t="n"/>
       <c r="G18" s="1" t="n"/>
       <c r="J18" t="n">
-        <v>204.3</v>
+        <v>5075.4</v>
       </c>
       <c r="K18" t="n">
-        <v>197.85</v>
+        <v>4998.05</v>
       </c>
       <c r="L18" t="n">
-        <v>5036.15</v>
+        <v>5021.25</v>
       </c>
       <c r="M18" t="n">
-        <v>5026.25</v>
+        <v>5012.3</v>
       </c>
       <c r="N18" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="O18" t="n">
-        <v>203.81</v>
+        <v>5022</v>
       </c>
     </row>
     <row r="19">
@@ -1953,22 +2031,22 @@
       <c r="F19" s="1" t="n"/>
       <c r="G19" s="1" t="n"/>
       <c r="J19" t="n">
-        <v>251.6</v>
+        <v>194.53</v>
       </c>
       <c r="K19" t="n">
-        <v>246.15</v>
+        <v>191.27</v>
       </c>
       <c r="L19" t="n">
-        <v>196.69</v>
+        <v>191.7</v>
       </c>
       <c r="M19" t="n">
-        <v>196.73</v>
+        <v>191.58</v>
       </c>
       <c r="N19" t="n">
-        <v>129</v>
+        <v>80</v>
       </c>
       <c r="O19" t="n">
-        <v>248.6</v>
+        <v>194.35</v>
       </c>
     </row>
     <row r="20">
@@ -1984,22 +2062,22 @@
       <c r="F20" s="1" t="n"/>
       <c r="G20" s="1" t="n"/>
       <c r="J20" t="n">
-        <v>513.45</v>
+        <v>1793.1</v>
       </c>
       <c r="K20" t="n">
-        <v>502.5</v>
+        <v>1750.05</v>
       </c>
       <c r="L20" t="n">
-        <v>1796</v>
+        <v>1789.45</v>
       </c>
       <c r="M20" t="n">
-        <v>1796.1</v>
+        <v>1788.9</v>
       </c>
       <c r="N20" t="n">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="O20" t="n">
-        <v>508.25</v>
+        <v>1751.15</v>
       </c>
     </row>
     <row r="21">
@@ -2015,22 +2093,22 @@
       <c r="F21" s="1" t="n"/>
       <c r="G21" s="1" t="n"/>
       <c r="J21" t="n">
-        <v>916.35</v>
+        <v>1645.85</v>
       </c>
       <c r="K21" t="n">
-        <v>893.05</v>
+        <v>1628.5</v>
       </c>
       <c r="L21" t="n">
-        <v>1732</v>
+        <v>1636.7</v>
       </c>
       <c r="M21" t="n">
-        <v>1732.05</v>
+        <v>1636.7</v>
       </c>
       <c r="N21" t="n">
-        <v>131</v>
+        <v>115</v>
       </c>
       <c r="O21" t="n">
-        <v>916.3</v>
+        <v>1645.3</v>
       </c>
     </row>
     <row r="22">
@@ -2046,22 +2124,22 @@
       <c r="F22" s="1" t="n"/>
       <c r="G22" s="1" t="n"/>
       <c r="J22" t="n">
-        <v>5085</v>
+        <v>619</v>
       </c>
       <c r="K22" t="n">
-        <v>4998.5</v>
+        <v>610</v>
       </c>
       <c r="L22" t="n">
-        <v>755</v>
+        <v>616</v>
       </c>
       <c r="M22" t="n">
-        <v>756.2</v>
+        <v>617</v>
       </c>
       <c r="N22" t="n">
-        <v>85</v>
+        <v>64</v>
       </c>
       <c r="O22" t="n">
-        <v>5050</v>
+        <v>610.95</v>
       </c>
     </row>
     <row r="23">
@@ -2077,22 +2155,22 @@
       <c r="F23" s="1" t="n"/>
       <c r="G23" s="1" t="n"/>
       <c r="J23" t="n">
-        <v>197.7</v>
+        <v>1240.95</v>
       </c>
       <c r="K23" t="n">
-        <v>192.9</v>
+        <v>1218</v>
       </c>
       <c r="L23" t="n">
-        <v>1273.95</v>
+        <v>1225.15</v>
       </c>
       <c r="M23" t="n">
-        <v>1273</v>
+        <v>1225.15</v>
       </c>
       <c r="N23" t="n">
-        <v>126</v>
+        <v>97</v>
       </c>
       <c r="O23" t="n">
-        <v>194.92</v>
+        <v>1239.45</v>
       </c>
     </row>
     <row r="24">
@@ -2108,22 +2186,22 @@
       <c r="F24" s="1" t="n"/>
       <c r="G24" s="1" t="n"/>
       <c r="J24" t="n">
-        <v>1820.7</v>
+        <v>975.6</v>
       </c>
       <c r="K24" t="n">
-        <v>1789.15</v>
+        <v>959</v>
       </c>
       <c r="L24" t="n">
-        <v>1445</v>
+        <v>972.9</v>
       </c>
       <c r="M24" t="n">
-        <v>1447.6</v>
+        <v>970.95</v>
       </c>
       <c r="N24" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="O24" t="n">
-        <v>1810.4</v>
+        <v>961.5</v>
       </c>
     </row>
     <row r="25">
@@ -2139,22 +2217,22 @@
       <c r="F25" s="1" t="n"/>
       <c r="G25" s="1" t="n"/>
       <c r="J25" t="n">
-        <v>1750.75</v>
+        <v>1851.1</v>
       </c>
       <c r="K25" t="n">
-        <v>1724.4</v>
+        <v>1812</v>
       </c>
       <c r="L25" t="n">
-        <v>1877.6</v>
+        <v>1817.5</v>
       </c>
       <c r="M25" t="n">
-        <v>1875.6</v>
+        <v>1815.45</v>
       </c>
       <c r="N25" t="n">
-        <v>69</v>
+        <v>164</v>
       </c>
       <c r="O25" t="n">
-        <v>1748.95</v>
+        <v>1844.55</v>
       </c>
     </row>
     <row r="26">
@@ -2170,22 +2248,22 @@
       <c r="F26" s="1" t="n"/>
       <c r="G26" s="1" t="n"/>
       <c r="J26" t="n">
-        <v>763.2</v>
+        <v>930.9</v>
       </c>
       <c r="K26" t="n">
-        <v>753.15</v>
+        <v>916.5</v>
       </c>
       <c r="L26" t="n">
-        <v>1038</v>
+        <v>924.9</v>
       </c>
       <c r="M26" t="n">
-        <v>1039.65</v>
+        <v>924.65</v>
       </c>
       <c r="N26" t="n">
-        <v>30</v>
+        <v>13</v>
       </c>
       <c r="O26" t="n">
-        <v>760.65</v>
+        <v>918</v>
       </c>
     </row>
     <row r="27">
@@ -2201,22 +2279,22 @@
       <c r="F27" s="1" t="n"/>
       <c r="G27" s="1" t="n"/>
       <c r="J27" t="n">
-        <v>1291.7</v>
+        <v>566.95</v>
       </c>
       <c r="K27" t="n">
-        <v>1270.9</v>
+        <v>557.25</v>
       </c>
       <c r="L27" t="n">
-        <v>662.9</v>
+        <v>562.95</v>
       </c>
       <c r="M27" t="n">
-        <v>662.45</v>
+        <v>562.7</v>
       </c>
       <c r="N27" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="O27" t="n">
-        <v>1289.2</v>
+        <v>562.6</v>
       </c>
     </row>
     <row r="28">
@@ -2232,22 +2310,22 @@
       <c r="F28" s="1" t="n"/>
       <c r="G28" s="1" t="n"/>
       <c r="J28" t="n">
-        <v>1455.9</v>
+        <v>2968.3</v>
       </c>
       <c r="K28" t="n">
-        <v>1437</v>
+        <v>2903.1</v>
       </c>
       <c r="L28" t="n">
-        <v>3115</v>
+        <v>2922.35</v>
       </c>
       <c r="M28" t="n">
-        <v>3094.9</v>
+        <v>2917</v>
       </c>
       <c r="N28" t="n">
-        <v>35</v>
+        <v>20</v>
       </c>
       <c r="O28" t="n">
-        <v>1455</v>
+        <v>2933.45</v>
       </c>
     </row>
     <row r="29">
@@ -2263,202 +2341,202 @@
       <c r="F29" s="1" t="n"/>
       <c r="G29" s="1" t="n"/>
       <c r="J29" t="n">
-        <v>1901.25</v>
+        <v>274.5</v>
       </c>
       <c r="K29" t="n">
-        <v>1870.5</v>
+        <v>267.75</v>
       </c>
       <c r="L29" t="n">
-        <v>340.35</v>
+        <v>268</v>
       </c>
       <c r="M29" t="n">
-        <v>338.35</v>
+        <v>268.55</v>
       </c>
       <c r="N29" t="n">
-        <v>49</v>
+        <v>11</v>
       </c>
       <c r="O29" t="n">
-        <v>1889.55</v>
+        <v>268.8</v>
       </c>
     </row>
     <row r="30">
       <c r="J30" t="n">
-        <v>1058.85</v>
+        <v>329</v>
       </c>
       <c r="K30" t="n">
-        <v>1023.55</v>
+        <v>325</v>
       </c>
       <c r="L30" t="n">
-        <v>443</v>
+        <v>326</v>
       </c>
       <c r="M30" t="n">
-        <v>443.2</v>
+        <v>326.15</v>
       </c>
       <c r="N30" t="n">
-        <v>209</v>
+        <v>71</v>
       </c>
       <c r="O30" t="n">
-        <v>1032.45</v>
+        <v>325.65</v>
       </c>
     </row>
     <row r="31">
       <c r="J31" t="n">
-        <v>670.55</v>
+        <v>1306.4</v>
       </c>
       <c r="K31" t="n">
-        <v>659.25</v>
+        <v>1285</v>
       </c>
       <c r="L31" t="n">
-        <v>2958</v>
+        <v>1300</v>
       </c>
       <c r="M31" t="n">
-        <v>2953.15</v>
+        <v>1302</v>
       </c>
       <c r="N31" t="n">
-        <v>135</v>
+        <v>293</v>
       </c>
       <c r="O31" t="n">
-        <v>662.8</v>
+        <v>1302.3</v>
       </c>
     </row>
     <row r="32">
       <c r="J32" t="n">
-        <v>3151.95</v>
+        <v>767.95</v>
       </c>
       <c r="K32" t="n">
-        <v>3087</v>
+        <v>759.4</v>
       </c>
       <c r="L32" t="n">
-        <v>788</v>
+        <v>763.8</v>
       </c>
       <c r="M32" t="n">
-        <v>787.9</v>
+        <v>764</v>
       </c>
       <c r="N32" t="n">
-        <v>154</v>
+        <v>57</v>
       </c>
       <c r="O32" t="n">
-        <v>3137.2</v>
+        <v>764.7</v>
       </c>
     </row>
     <row r="33">
       <c r="J33" t="n">
-        <v>341.65</v>
+        <v>658.5</v>
       </c>
       <c r="K33" t="n">
-        <v>330.65</v>
+        <v>648</v>
       </c>
       <c r="L33" t="n">
-        <v>833.5</v>
+        <v>653.4</v>
       </c>
       <c r="M33" t="n">
-        <v>833.1</v>
+        <v>649.35</v>
       </c>
       <c r="N33" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O33" t="n">
-        <v>334.75</v>
+        <v>654</v>
       </c>
     </row>
     <row r="34">
       <c r="J34" t="n">
-        <v>445.95</v>
+        <v>986.95</v>
       </c>
       <c r="K34" t="n">
-        <v>433.6</v>
+        <v>968.75</v>
       </c>
       <c r="L34" t="n">
-        <v>1091.5</v>
+        <v>974</v>
       </c>
       <c r="M34" t="n">
-        <v>1091.1</v>
+        <v>975.35</v>
       </c>
       <c r="N34" t="n">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="O34" t="n">
-        <v>444.4</v>
+        <v>984.7</v>
       </c>
     </row>
     <row r="35">
       <c r="J35" t="n">
-        <v>3027.5</v>
+        <v>785.5</v>
       </c>
       <c r="K35" t="n">
-        <v>2948.8</v>
+        <v>774.6</v>
       </c>
       <c r="L35" t="n">
-        <v>975.8</v>
+        <v>779.9</v>
       </c>
       <c r="M35" t="n">
-        <v>974.65</v>
+        <v>779.65</v>
       </c>
       <c r="N35" t="n">
-        <v>122</v>
+        <v>70</v>
       </c>
       <c r="O35" t="n">
-        <v>3025.35</v>
+        <v>776.55</v>
       </c>
     </row>
     <row r="36">
       <c r="J36" t="n">
-        <v>799.3</v>
+        <v>375.4</v>
       </c>
       <c r="K36" t="n">
-        <v>786.45</v>
+        <v>366.4</v>
       </c>
       <c r="L36" t="n">
-        <v>482.5</v>
+        <v>373.5</v>
       </c>
       <c r="M36" t="n">
-        <v>482.6</v>
+        <v>373.6</v>
       </c>
       <c r="N36" t="n">
-        <v>157</v>
+        <v>55</v>
       </c>
       <c r="O36" t="n">
-        <v>798.8</v>
+        <v>367.3</v>
       </c>
     </row>
     <row r="37">
       <c r="J37" t="n">
-        <v>837.95</v>
+        <v>131.16</v>
       </c>
       <c r="K37" t="n">
-        <v>824.4</v>
+        <v>127.66</v>
       </c>
       <c r="L37" t="n">
-        <v>168.11</v>
+        <v>130.15</v>
       </c>
       <c r="M37" t="n">
-        <v>168.55</v>
+        <v>130.28</v>
       </c>
       <c r="N37" t="n">
-        <v>923</v>
+        <v>274</v>
       </c>
       <c r="O37" t="n">
-        <v>832.95</v>
+        <v>127.94</v>
       </c>
     </row>
     <row r="38">
       <c r="J38" t="n">
-        <v>1101.3</v>
+        <v>10723.95</v>
       </c>
       <c r="K38" t="n">
-        <v>1074.15</v>
+        <v>10500.1</v>
       </c>
       <c r="L38" t="n">
-        <v>11800</v>
+        <v>10600</v>
       </c>
       <c r="M38" t="n">
-        <v>11802</v>
+        <v>10580</v>
       </c>
       <c r="N38" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O38" t="n">
-        <v>1092.15</v>
+        <v>10639.7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Changed bn row & fixed closing dates in MWCL
</commit_message>
<xml_diff>
--- a/cash high low.xlsx
+++ b/cash high low.xlsx
@@ -78,7 +78,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="23">
+  <borders count="22">
     <border>
       <left/>
       <right/>
@@ -322,19 +322,6 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left style="thin">
         <color indexed="64"/>
       </left>
@@ -367,7 +354,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="2" pivotButton="0" quotePrefix="0" xfId="1"/>
@@ -393,11 +380,9 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="11" pivotButton="0" quotePrefix="0" xfId="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="12" pivotButton="0" quotePrefix="0" xfId="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="9" pivotButton="0" quotePrefix="0" xfId="1"/>
-    <xf numFmtId="3" fontId="4" fillId="0" borderId="20" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="21" pivotButton="0" quotePrefix="0" xfId="1"/>
-    <xf numFmtId="2" fontId="2" fillId="2" borderId="22" pivotButton="0" quotePrefix="0" xfId="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="21" pivotButton="0" quotePrefix="0" xfId="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="21" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="2" fillId="2" borderId="21" pivotButton="0" quotePrefix="0" xfId="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="20" pivotButton="0" quotePrefix="0" xfId="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="2" fillId="2" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment horizontal="right"/>
@@ -827,22 +812,22 @@
         </is>
       </c>
       <c r="B2" s="19" t="n">
-        <v>446.5</v>
+        <v>398.45</v>
       </c>
       <c r="C2" s="16" t="n">
-        <v>438.6</v>
+        <v>388.25</v>
       </c>
       <c r="D2" s="6" t="n">
-        <v>446.5</v>
-      </c>
-      <c r="E2" s="31" t="n">
-        <v>444.7</v>
+        <v>393</v>
+      </c>
+      <c r="E2" s="29" t="n">
+        <v>392.65</v>
       </c>
       <c r="F2" s="8" t="n">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>442</v>
+        <v>394.3</v>
       </c>
     </row>
     <row r="3">
@@ -852,22 +837,22 @@
         </is>
       </c>
       <c r="B3" s="19" t="n">
-        <v>2314.95</v>
+        <v>2267.85</v>
       </c>
       <c r="C3" s="16" t="n">
-        <v>2238.4</v>
+        <v>2233.05</v>
       </c>
       <c r="D3" s="6" t="n">
-        <v>2297</v>
-      </c>
-      <c r="E3" s="31" t="n">
-        <v>2287.8</v>
+        <v>2252.65</v>
+      </c>
+      <c r="E3" s="29" t="n">
+        <v>2250.6</v>
       </c>
       <c r="F3" s="8" t="n">
-        <v>20</v>
+        <v>9</v>
       </c>
       <c r="G3" s="4" t="n">
-        <v>2241.7</v>
+        <v>2240.85</v>
       </c>
     </row>
     <row r="4">
@@ -877,22 +862,22 @@
         </is>
       </c>
       <c r="B4" s="20" t="n">
-        <v>439.1</v>
+        <v>407</v>
       </c>
       <c r="C4" s="17" t="n">
-        <v>431.8</v>
+        <v>401.05</v>
       </c>
       <c r="D4" s="7" t="n">
-        <v>437.05</v>
-      </c>
-      <c r="E4" s="32" t="n">
-        <v>437.3</v>
+        <v>402.95</v>
+      </c>
+      <c r="E4" s="30" t="n">
+        <v>402.1</v>
       </c>
       <c r="F4" s="9" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="G4" s="5" t="n">
-        <v>433.8</v>
+        <v>405.8</v>
       </c>
     </row>
     <row r="5">
@@ -902,22 +887,22 @@
         </is>
       </c>
       <c r="B5" s="20" t="n">
-        <v>1753.7</v>
+        <v>1827.65</v>
       </c>
       <c r="C5" s="17" t="n">
-        <v>1698.2</v>
+        <v>1788.25</v>
       </c>
       <c r="D5" s="7" t="n">
-        <v>1742.35</v>
-      </c>
-      <c r="E5" s="32" t="n">
-        <v>1736.1</v>
+        <v>1808.2</v>
+      </c>
+      <c r="E5" s="30" t="n">
+        <v>1805.4</v>
       </c>
       <c r="F5" s="9" t="n">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="G5" s="5" t="n">
-        <v>1720.2</v>
+        <v>1822.4</v>
       </c>
     </row>
     <row r="6">
@@ -927,22 +912,22 @@
         </is>
       </c>
       <c r="B6" s="20" t="n">
-        <v>7980.65</v>
+        <v>8375</v>
       </c>
       <c r="C6" s="17" t="n">
-        <v>7791</v>
+        <v>8250</v>
       </c>
       <c r="D6" s="7" t="n">
-        <v>7898.75</v>
-      </c>
-      <c r="E6" s="32" t="n">
-        <v>7885.1</v>
+        <v>8344.9</v>
+      </c>
+      <c r="E6" s="30" t="n">
+        <v>8340.450000000001</v>
       </c>
       <c r="F6" s="9" t="n">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="G6" s="5" t="n">
-        <v>7860.6</v>
+        <v>8295</v>
       </c>
     </row>
     <row r="7">
@@ -952,22 +937,22 @@
         </is>
       </c>
       <c r="B7" s="20" t="n">
-        <v>152.59</v>
+        <v>142.88</v>
       </c>
       <c r="C7" s="17" t="n">
-        <v>147.35</v>
+        <v>138.27</v>
       </c>
       <c r="D7" s="7" t="n">
-        <v>151.6</v>
-      </c>
-      <c r="E7" s="32" t="n">
-        <v>151.38</v>
+        <v>140.63</v>
+      </c>
+      <c r="E7" s="30" t="n">
+        <v>140.11</v>
       </c>
       <c r="F7" s="9" t="n">
-        <v>67</v>
+        <v>226</v>
       </c>
       <c r="G7" s="5" t="n">
-        <v>148.25</v>
+        <v>141.5</v>
       </c>
     </row>
     <row r="8">
@@ -977,22 +962,22 @@
         </is>
       </c>
       <c r="B8" s="20" t="n">
-        <v>217.13</v>
+        <v>204.8</v>
       </c>
       <c r="C8" s="17" t="n">
-        <v>211.05</v>
+        <v>201.58</v>
       </c>
       <c r="D8" s="7" t="n">
-        <v>213.61</v>
-      </c>
-      <c r="E8" s="32" t="n">
-        <v>213.39</v>
+        <v>202.7</v>
+      </c>
+      <c r="E8" s="30" t="n">
+        <v>202.56</v>
       </c>
       <c r="F8" s="9" t="n">
-        <v>508</v>
+        <v>129</v>
       </c>
       <c r="G8" s="5" t="n">
-        <v>214.88</v>
+        <v>203.48</v>
       </c>
     </row>
     <row r="9">
@@ -1002,22 +987,22 @@
         </is>
       </c>
       <c r="B9" s="20" t="n">
-        <v>396.95</v>
+        <v>380</v>
       </c>
       <c r="C9" s="17" t="n">
-        <v>378.15</v>
+        <v>371.7</v>
       </c>
       <c r="D9" s="7" t="n">
-        <v>396.5</v>
-      </c>
-      <c r="E9" s="32" t="n">
-        <v>395.9</v>
+        <v>378.6</v>
+      </c>
+      <c r="E9" s="30" t="n">
+        <v>379.05</v>
       </c>
       <c r="F9" s="9" t="n">
-        <v>103</v>
+        <v>53</v>
       </c>
       <c r="G9" s="5" t="n">
-        <v>380.35</v>
+        <v>375.25</v>
       </c>
     </row>
     <row r="10">
@@ -1027,22 +1012,22 @@
         </is>
       </c>
       <c r="B10" s="20" t="n">
-        <v>754</v>
+        <v>674.95</v>
       </c>
       <c r="C10" s="17" t="n">
-        <v>738</v>
+        <v>641.55</v>
       </c>
       <c r="D10" s="7" t="n">
-        <v>745</v>
-      </c>
-      <c r="E10" s="32" t="n">
-        <v>745.05</v>
+        <v>674</v>
+      </c>
+      <c r="E10" s="30" t="n">
+        <v>674.1</v>
       </c>
       <c r="F10" s="9" t="n">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="G10" s="5" t="n">
-        <v>744</v>
+        <v>645.8</v>
       </c>
     </row>
     <row r="11">
@@ -1052,22 +1037,22 @@
         </is>
       </c>
       <c r="B11" s="20" t="n">
-        <v>5244</v>
+        <v>5010</v>
       </c>
       <c r="C11" s="17" t="n">
-        <v>5154.5</v>
+        <v>4912.05</v>
       </c>
       <c r="D11" s="7" t="n">
-        <v>5198.25</v>
-      </c>
-      <c r="E11" s="32" t="n">
-        <v>5194.3</v>
+        <v>5005</v>
+      </c>
+      <c r="E11" s="30" t="n">
+        <v>4985.55</v>
       </c>
       <c r="F11" s="9" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G11" s="5" t="n">
-        <v>5172.7</v>
+        <v>4975.6</v>
       </c>
     </row>
     <row r="12">
@@ -1077,22 +1062,22 @@
         </is>
       </c>
       <c r="B12" s="20" t="n">
-        <v>188.28</v>
+        <v>180.25</v>
       </c>
       <c r="C12" s="17" t="n">
-        <v>185.7</v>
+        <v>175.5</v>
       </c>
       <c r="D12" s="7" t="n">
-        <v>187.1</v>
-      </c>
-      <c r="E12" s="32" t="n">
-        <v>187.21</v>
+        <v>179.2</v>
+      </c>
+      <c r="E12" s="30" t="n">
+        <v>179.12</v>
       </c>
       <c r="F12" s="9" t="n">
         <v>57</v>
       </c>
       <c r="G12" s="5" t="n">
-        <v>185.97</v>
+        <v>176.83</v>
       </c>
     </row>
     <row r="13">
@@ -1102,22 +1087,22 @@
         </is>
       </c>
       <c r="B13" s="20" t="n">
-        <v>1738.2</v>
+        <v>1573.95</v>
       </c>
       <c r="C13" s="17" t="n">
-        <v>1713</v>
+        <v>1535.5</v>
       </c>
       <c r="D13" s="7" t="n">
-        <v>1730</v>
-      </c>
-      <c r="E13" s="32" t="n">
-        <v>1725.45</v>
+        <v>1567</v>
+      </c>
+      <c r="E13" s="30" t="n">
+        <v>1567.85</v>
       </c>
       <c r="F13" s="9" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="G13" s="5" t="n">
-        <v>1726.05</v>
+        <v>1542.1</v>
       </c>
     </row>
     <row r="14">
@@ -1127,22 +1112,22 @@
         </is>
       </c>
       <c r="B14" s="20" t="n">
-        <v>1704.7</v>
+        <v>1694</v>
       </c>
       <c r="C14" s="17" t="n">
-        <v>1683.95</v>
+        <v>1670.65</v>
       </c>
       <c r="D14" s="7" t="n">
-        <v>1699.5</v>
-      </c>
-      <c r="E14" s="32" t="n">
-        <v>1698.75</v>
+        <v>1687.9</v>
+      </c>
+      <c r="E14" s="30" t="n">
+        <v>1685.5</v>
       </c>
       <c r="F14" s="9" t="n">
-        <v>79</v>
+        <v>99</v>
       </c>
       <c r="G14" s="5" t="n">
-        <v>1686.6</v>
+        <v>1671.4</v>
       </c>
     </row>
     <row r="15">
@@ -1152,22 +1137,22 @@
         </is>
       </c>
       <c r="B15" s="20" t="n">
-        <v>596.4</v>
+        <v>699</v>
       </c>
       <c r="C15" s="17" t="n">
-        <v>585.1</v>
+        <v>685.1</v>
       </c>
       <c r="D15" s="7" t="n">
-        <v>593.75</v>
-      </c>
-      <c r="E15" s="32" t="n">
-        <v>594.3</v>
+        <v>699</v>
+      </c>
+      <c r="E15" s="30" t="n">
+        <v>695.5</v>
       </c>
       <c r="F15" s="9" t="n">
-        <v>37</v>
+        <v>52</v>
       </c>
       <c r="G15" s="5" t="n">
-        <v>587.5</v>
+        <v>688.35</v>
       </c>
     </row>
     <row r="16">
@@ -1177,22 +1162,22 @@
         </is>
       </c>
       <c r="B16" s="20" t="n">
-        <v>1255</v>
+        <v>1248</v>
       </c>
       <c r="C16" s="17" t="n">
-        <v>1239.1</v>
+        <v>1223.8</v>
       </c>
       <c r="D16" s="7" t="n">
-        <v>1252.95</v>
-      </c>
-      <c r="E16" s="32" t="n">
-        <v>1252.8</v>
+        <v>1244.15</v>
+      </c>
+      <c r="E16" s="30" t="n">
+        <v>1245.4</v>
       </c>
       <c r="F16" s="9" t="n">
-        <v>101</v>
+        <v>109</v>
       </c>
       <c r="G16" s="5" t="n">
-        <v>1246.05</v>
+        <v>1225.55</v>
       </c>
     </row>
     <row r="17">
@@ -1202,22 +1187,22 @@
         </is>
       </c>
       <c r="B17" s="20" t="n">
-        <v>999.3</v>
+        <v>810.45</v>
       </c>
       <c r="C17" s="17" t="n">
-        <v>953.85</v>
+        <v>649</v>
       </c>
       <c r="D17" s="7" t="n">
-        <v>995.2</v>
-      </c>
-      <c r="E17" s="32" t="n">
-        <v>991.2</v>
+        <v>656.8</v>
+      </c>
+      <c r="E17" s="30" t="n">
+        <v>655.95</v>
       </c>
       <c r="F17" s="9" t="n">
-        <v>53</v>
+        <v>1010</v>
       </c>
       <c r="G17" s="5" t="n">
-        <v>962.75</v>
+        <v>810.45</v>
       </c>
     </row>
     <row r="18">
@@ -1227,22 +1212,22 @@
         </is>
       </c>
       <c r="B18" s="20" t="n">
-        <v>1894.55</v>
+        <v>1668</v>
       </c>
       <c r="C18" s="17" t="n">
-        <v>1875.05</v>
+        <v>1637.05</v>
       </c>
       <c r="D18" s="7" t="n">
-        <v>1882.95</v>
-      </c>
-      <c r="E18" s="32" t="n">
-        <v>1879.8</v>
+        <v>1667</v>
+      </c>
+      <c r="E18" s="30" t="n">
+        <v>1661.6</v>
       </c>
       <c r="F18" s="9" t="n">
-        <v>58</v>
+        <v>126</v>
       </c>
       <c r="G18" s="5" t="n">
-        <v>1884.4</v>
+        <v>1659.45</v>
       </c>
     </row>
     <row r="19">
@@ -1252,22 +1237,22 @@
         </is>
       </c>
       <c r="B19" s="20" t="n">
-        <v>796.8</v>
+        <v>909.5</v>
       </c>
       <c r="C19" s="17" t="n">
-        <v>723.35</v>
+        <v>894.35</v>
       </c>
       <c r="D19" s="7" t="n">
-        <v>787.7</v>
-      </c>
-      <c r="E19" s="32" t="n">
-        <v>791.55</v>
+        <v>907.1</v>
+      </c>
+      <c r="E19" s="30" t="n">
+        <v>904.85</v>
       </c>
       <c r="F19" s="9" t="n">
-        <v>226</v>
+        <v>27</v>
       </c>
       <c r="G19" s="5" t="n">
-        <v>756.05</v>
+        <v>903.25</v>
       </c>
     </row>
     <row r="20">
@@ -1277,22 +1262,22 @@
         </is>
       </c>
       <c r="B20" s="20" t="n">
-        <v>601.45</v>
+        <v>535.65</v>
       </c>
       <c r="C20" s="17" t="n">
-        <v>570.25</v>
+        <v>519.65</v>
       </c>
       <c r="D20" s="7" t="n">
-        <v>600</v>
-      </c>
-      <c r="E20" s="32" t="n">
-        <v>598.1</v>
+        <v>535</v>
+      </c>
+      <c r="E20" s="30" t="n">
+        <v>533.6</v>
       </c>
       <c r="F20" s="9" t="n">
-        <v>30</v>
+        <v>14</v>
       </c>
       <c r="G20" s="5" t="n">
-        <v>582.9</v>
+        <v>523.8</v>
       </c>
     </row>
     <row r="21">
@@ -1302,22 +1287,22 @@
         </is>
       </c>
       <c r="B21" s="20" t="n">
-        <v>3049.85</v>
+        <v>2674</v>
       </c>
       <c r="C21" s="17" t="n">
-        <v>2985.25</v>
+        <v>2613.15</v>
       </c>
       <c r="D21" s="7" t="n">
-        <v>3000</v>
-      </c>
-      <c r="E21" s="32" t="n">
-        <v>2989.85</v>
+        <v>2657.85</v>
+      </c>
+      <c r="E21" s="30" t="n">
+        <v>2645.6</v>
       </c>
       <c r="F21" s="9" t="n">
-        <v>24</v>
+        <v>36</v>
       </c>
       <c r="G21" s="5" t="n">
-        <v>3000.65</v>
+        <v>2646.7</v>
       </c>
     </row>
     <row r="22">
@@ -1327,22 +1312,22 @@
         </is>
       </c>
       <c r="B22" s="20" t="n">
-        <v>285.8</v>
+        <v>271.4</v>
       </c>
       <c r="C22" s="17" t="n">
-        <v>277</v>
+        <v>265.3</v>
       </c>
       <c r="D22" s="7" t="n">
-        <v>285.1</v>
-      </c>
-      <c r="E22" s="32" t="n">
-        <v>284.95</v>
+        <v>269.7</v>
+      </c>
+      <c r="E22" s="30" t="n">
+        <v>268.6</v>
       </c>
       <c r="F22" s="9" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="G22" s="5" t="n">
-        <v>278.1</v>
+        <v>268.7</v>
       </c>
     </row>
     <row r="23">
@@ -1352,22 +1337,22 @@
         </is>
       </c>
       <c r="B23" s="20" t="n">
-        <v>326.25</v>
+        <v>333.25</v>
       </c>
       <c r="C23" s="17" t="n">
-        <v>319.1</v>
+        <v>327.25</v>
       </c>
       <c r="D23" s="7" t="n">
-        <v>325.15</v>
-      </c>
-      <c r="E23" s="32" t="n">
-        <v>324</v>
+        <v>331.5</v>
+      </c>
+      <c r="E23" s="30" t="n">
+        <v>330.3</v>
       </c>
       <c r="F23" s="9" t="n">
-        <v>131</v>
+        <v>102</v>
       </c>
       <c r="G23" s="5" t="n">
-        <v>319.8</v>
+        <v>329.7</v>
       </c>
     </row>
     <row r="24">
@@ -1377,22 +1362,22 @@
         </is>
       </c>
       <c r="B24" s="20" t="n">
-        <v>1267</v>
+        <v>1249.5</v>
       </c>
       <c r="C24" s="17" t="n">
-        <v>1251.75</v>
+        <v>1230.8</v>
       </c>
       <c r="D24" s="7" t="n">
-        <v>1266</v>
-      </c>
-      <c r="E24" s="32" t="n">
-        <v>1265.1</v>
+        <v>1247.25</v>
+      </c>
+      <c r="E24" s="30" t="n">
+        <v>1247.3</v>
       </c>
       <c r="F24" s="9" t="n">
-        <v>65</v>
+        <v>100</v>
       </c>
       <c r="G24" s="5" t="n">
-        <v>1254.25</v>
+        <v>1231.45</v>
       </c>
     </row>
     <row r="25">
@@ -1402,22 +1387,22 @@
         </is>
       </c>
       <c r="B25" s="20" t="n">
-        <v>777.55</v>
+        <v>734.05</v>
       </c>
       <c r="C25" s="17" t="n">
-        <v>760</v>
+        <v>724.95</v>
       </c>
       <c r="D25" s="7" t="n">
-        <v>773.1</v>
-      </c>
-      <c r="E25" s="32" t="n">
-        <v>772.9</v>
+        <v>729.9</v>
+      </c>
+      <c r="E25" s="30" t="n">
+        <v>729.85</v>
       </c>
       <c r="F25" s="9" t="n">
-        <v>100</v>
+        <v>55</v>
       </c>
       <c r="G25" s="5" t="n">
-        <v>763.1</v>
+        <v>726.45</v>
       </c>
     </row>
     <row r="26">
@@ -1427,22 +1412,22 @@
         </is>
       </c>
       <c r="B26" s="20" t="n">
-        <v>635.8</v>
+        <v>582.6</v>
       </c>
       <c r="C26" s="17" t="n">
-        <v>613.6</v>
+        <v>555.4</v>
       </c>
       <c r="D26" s="7" t="n">
-        <v>619</v>
-      </c>
-      <c r="E26" s="32" t="n">
-        <v>618.85</v>
+        <v>577.1</v>
+      </c>
+      <c r="E26" s="30" t="n">
+        <v>579.2</v>
       </c>
       <c r="F26" s="9" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G26" s="5" t="n">
-        <v>634.65</v>
+        <v>556.7</v>
       </c>
     </row>
     <row r="27">
@@ -1452,22 +1437,22 @@
         </is>
       </c>
       <c r="B27" s="20" t="n">
-        <v>990</v>
+        <v>825.5</v>
       </c>
       <c r="C27" s="17" t="n">
-        <v>968.05</v>
+        <v>804.4</v>
       </c>
       <c r="D27" s="7" t="n">
-        <v>983</v>
-      </c>
-      <c r="E27" s="32" t="n">
-        <v>986.1</v>
+        <v>817</v>
+      </c>
+      <c r="E27" s="30" t="n">
+        <v>815.9</v>
       </c>
       <c r="F27" s="9" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G27" s="5" t="n">
-        <v>971.65</v>
+        <v>813.4</v>
       </c>
     </row>
     <row r="28">
@@ -1477,22 +1462,22 @@
         </is>
       </c>
       <c r="B28" s="20" t="n">
-        <v>717</v>
+        <v>651.15</v>
       </c>
       <c r="C28" s="17" t="n">
-        <v>699.55</v>
+        <v>642.5</v>
       </c>
       <c r="D28" s="7" t="n">
-        <v>715.7</v>
-      </c>
-      <c r="E28" s="32" t="n">
-        <v>716.1</v>
+        <v>648.9</v>
+      </c>
+      <c r="E28" s="30" t="n">
+        <v>648.05</v>
       </c>
       <c r="F28" s="9" t="n">
-        <v>191</v>
+        <v>95</v>
       </c>
       <c r="G28" s="5" t="n">
-        <v>703.65</v>
+        <v>646.95</v>
       </c>
     </row>
     <row r="29">
@@ -1502,22 +1487,22 @@
         </is>
       </c>
       <c r="B29" s="20" t="n">
-        <v>366.95</v>
+        <v>354</v>
       </c>
       <c r="C29" s="17" t="n">
-        <v>352.1</v>
+        <v>347.1</v>
       </c>
       <c r="D29" s="7" t="n">
-        <v>366.85</v>
-      </c>
-      <c r="E29" s="32" t="n">
-        <v>364.5</v>
+        <v>353.75</v>
+      </c>
+      <c r="E29" s="30" t="n">
+        <v>352.45</v>
       </c>
       <c r="F29" s="22" t="n">
-        <v>70</v>
+        <v>51</v>
       </c>
       <c r="G29" s="23" t="n">
-        <v>353.65</v>
+        <v>350.45</v>
       </c>
     </row>
     <row r="30">
@@ -1527,22 +1512,22 @@
         </is>
       </c>
       <c r="B30" s="21" t="n">
-        <v>135</v>
+        <v>151.7</v>
       </c>
       <c r="C30" s="18" t="n">
-        <v>131.12</v>
+        <v>149.05</v>
       </c>
       <c r="D30" s="11" t="n">
-        <v>134.9</v>
-      </c>
-      <c r="E30" s="33" t="n">
-        <v>134.62</v>
+        <v>150.83</v>
+      </c>
+      <c r="E30" s="31" t="n">
+        <v>150.75</v>
       </c>
       <c r="F30" s="24" t="n">
-        <v>266</v>
+        <v>359</v>
       </c>
       <c r="G30" s="24" t="n">
-        <v>131.3</v>
+        <v>150.64</v>
       </c>
     </row>
     <row r="31" ht="15.75" customHeight="1" thickBot="1">
@@ -1551,23 +1536,23 @@
           <t>ULTRA</t>
         </is>
       </c>
-      <c r="B31" s="26" t="n">
-        <v>11599</v>
-      </c>
-      <c r="C31" s="25" t="n">
-        <v>11414.45</v>
-      </c>
-      <c r="D31" s="27" t="n">
-        <v>11599</v>
-      </c>
-      <c r="E31" s="34" t="n">
-        <v>11487.45</v>
-      </c>
-      <c r="F31" s="28" t="n">
-        <v>3</v>
-      </c>
-      <c r="G31" s="29" t="n">
-        <v>11434</v>
+      <c r="B31" s="21" t="n">
+        <v>10508.55</v>
+      </c>
+      <c r="C31" s="18" t="n">
+        <v>10356.25</v>
+      </c>
+      <c r="D31" s="25" t="n">
+        <v>10458.6</v>
+      </c>
+      <c r="E31" s="32" t="n">
+        <v>10439.25</v>
+      </c>
+      <c r="F31" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="G31" s="27" t="n">
+        <v>10436.75</v>
       </c>
     </row>
   </sheetData>
@@ -1711,7 +1696,7 @@
       <c r="E8" s="1" t="n"/>
       <c r="F8" s="1" t="n"/>
       <c r="G8" s="1" t="n"/>
-      <c r="J8" s="30" t="n">
+      <c r="J8" s="28" t="n">
         <v>45309</v>
       </c>
     </row>

</xml_diff>

<commit_message>
added 15 min sheets like 30 mins in net trader auto and 30 min cash, removed unused idx
</commit_message>
<xml_diff>
--- a/cash high low.xlsx
+++ b/cash high low.xlsx
@@ -818,22 +818,22 @@
         </is>
       </c>
       <c r="B2" s="19" t="n">
-        <v>472.5</v>
+        <v>387.25</v>
       </c>
       <c r="C2" s="16" t="n">
-        <v>466.15</v>
+        <v>383.2</v>
       </c>
       <c r="D2" s="6" t="n">
-        <v>468.75</v>
+        <v>386.5</v>
       </c>
       <c r="E2" s="29" t="n">
-        <v>468.1</v>
+        <v>385.45</v>
       </c>
       <c r="F2" s="8" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>471.8</v>
+        <v>384.8</v>
       </c>
     </row>
     <row r="3">
@@ -843,22 +843,22 @@
         </is>
       </c>
       <c r="B3" s="19" t="n">
-        <v>2567</v>
+        <v>2293</v>
       </c>
       <c r="C3" s="16" t="n">
-        <v>2541.3</v>
+        <v>2263.1</v>
       </c>
       <c r="D3" s="6" t="n">
-        <v>2543.6</v>
+        <v>2292</v>
       </c>
       <c r="E3" s="29" t="n">
-        <v>2547.7</v>
+        <v>2288.7</v>
       </c>
       <c r="F3" s="8" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G3" s="4" t="n">
-        <v>2558</v>
+        <v>2283.1</v>
       </c>
     </row>
     <row r="4">
@@ -868,22 +868,22 @@
         </is>
       </c>
       <c r="B4" s="20" t="n">
-        <v>500.55</v>
+        <v>495.7</v>
       </c>
       <c r="C4" s="17" t="n">
-        <v>489.5</v>
+        <v>482.4</v>
       </c>
       <c r="D4" s="7" t="n">
-        <v>497</v>
+        <v>486.1</v>
       </c>
       <c r="E4" s="30" t="n">
-        <v>495.15</v>
+        <v>485.65</v>
       </c>
       <c r="F4" s="9" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="G4" s="5" t="n">
-        <v>489.65</v>
+        <v>491.5</v>
       </c>
     </row>
     <row r="5">
@@ -893,22 +893,22 @@
         </is>
       </c>
       <c r="B5" s="20" t="n">
-        <v>2070</v>
+        <v>1972</v>
       </c>
       <c r="C5" s="17" t="n">
-        <v>2046</v>
+        <v>1950.8</v>
       </c>
       <c r="D5" s="7" t="n">
-        <v>2050.9</v>
+        <v>1971</v>
       </c>
       <c r="E5" s="30" t="n">
-        <v>2052.6</v>
+        <v>1966.1</v>
       </c>
       <c r="F5" s="9" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="G5" s="5" t="n">
-        <v>2055.1</v>
+        <v>1955.6</v>
       </c>
     </row>
     <row r="6">
@@ -918,22 +918,22 @@
         </is>
       </c>
       <c r="B6" s="20" t="n">
-        <v>9336.5</v>
+        <v>898.85</v>
       </c>
       <c r="C6" s="17" t="n">
-        <v>9250</v>
+        <v>883.6</v>
       </c>
       <c r="D6" s="7" t="n">
-        <v>9262</v>
+        <v>896.8</v>
       </c>
       <c r="E6" s="30" t="n">
-        <v>9269.5</v>
+        <v>896.3</v>
       </c>
       <c r="F6" s="9" t="n">
-        <v>5</v>
+        <v>54</v>
       </c>
       <c r="G6" s="5" t="n">
-        <v>9298</v>
+        <v>884.6</v>
       </c>
     </row>
     <row r="7">
@@ -943,22 +943,22 @@
         </is>
       </c>
       <c r="B7" s="20" t="n">
-        <v>166.68</v>
+        <v>165.47</v>
       </c>
       <c r="C7" s="17" t="n">
-        <v>164.4</v>
+        <v>163.25</v>
       </c>
       <c r="D7" s="7" t="n">
-        <v>165.46</v>
+        <v>164.95</v>
       </c>
       <c r="E7" s="30" t="n">
-        <v>165.62</v>
+        <v>164.73</v>
       </c>
       <c r="F7" s="9" t="n">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="G7" s="5" t="n">
-        <v>166.15</v>
+        <v>163.5</v>
       </c>
     </row>
     <row r="8">
@@ -968,22 +968,22 @@
         </is>
       </c>
       <c r="B8" s="20" t="n">
-        <v>244.85</v>
+        <v>239.07</v>
       </c>
       <c r="C8" s="17" t="n">
-        <v>240.8</v>
+        <v>237.12</v>
       </c>
       <c r="D8" s="7" t="n">
-        <v>241.47</v>
+        <v>238.4</v>
       </c>
       <c r="E8" s="30" t="n">
-        <v>241.52</v>
+        <v>238.42</v>
       </c>
       <c r="F8" s="9" t="n">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="G8" s="5" t="n">
-        <v>244.43</v>
+        <v>238.19</v>
       </c>
     </row>
     <row r="9">
@@ -993,22 +993,22 @@
         </is>
       </c>
       <c r="B9" s="20" t="n">
-        <v>405.8</v>
+        <v>393.3</v>
       </c>
       <c r="C9" s="17" t="n">
-        <v>401.75</v>
+        <v>380</v>
       </c>
       <c r="D9" s="7" t="n">
-        <v>402.4</v>
+        <v>389.4</v>
       </c>
       <c r="E9" s="30" t="n">
-        <v>402.7</v>
+        <v>389.8</v>
       </c>
       <c r="F9" s="9" t="n">
-        <v>60</v>
+        <v>81</v>
       </c>
       <c r="G9" s="5" t="n">
-        <v>403.1</v>
+        <v>381.4</v>
       </c>
     </row>
     <row r="10">
@@ -1018,22 +1018,22 @@
         </is>
       </c>
       <c r="B10" s="20" t="n">
-        <v>790.5</v>
+        <v>765.85</v>
       </c>
       <c r="C10" s="17" t="n">
-        <v>775</v>
+        <v>757</v>
       </c>
       <c r="D10" s="7" t="n">
-        <v>775.8</v>
+        <v>764.95</v>
       </c>
       <c r="E10" s="30" t="n">
-        <v>777.8</v>
+        <v>764.4</v>
       </c>
       <c r="F10" s="9" t="n">
-        <v>37</v>
+        <v>14</v>
       </c>
       <c r="G10" s="5" t="n">
-        <v>775</v>
+        <v>757.2</v>
       </c>
     </row>
     <row r="11">
@@ -1043,22 +1043,22 @@
         </is>
       </c>
       <c r="B11" s="20" t="n">
-        <v>5473</v>
+        <v>6379</v>
       </c>
       <c r="C11" s="17" t="n">
-        <v>5412</v>
+        <v>6308</v>
       </c>
       <c r="D11" s="7" t="n">
-        <v>5430</v>
+        <v>6374.5</v>
       </c>
       <c r="E11" s="30" t="n">
-        <v>5427.5</v>
+        <v>6371.5</v>
       </c>
       <c r="F11" s="9" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G11" s="5" t="n">
-        <v>5456</v>
+        <v>6323</v>
       </c>
     </row>
     <row r="12">
@@ -1068,22 +1068,22 @@
         </is>
       </c>
       <c r="B12" s="20" t="n">
-        <v>203.91</v>
+        <v>194.67</v>
       </c>
       <c r="C12" s="17" t="n">
-        <v>200.51</v>
+        <v>192.76</v>
       </c>
       <c r="D12" s="7" t="n">
-        <v>201.96</v>
+        <v>193.7</v>
       </c>
       <c r="E12" s="30" t="n">
-        <v>201.9</v>
+        <v>193.23</v>
       </c>
       <c r="F12" s="9" t="n">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="G12" s="5" t="n">
-        <v>203.66</v>
+        <v>193.65</v>
       </c>
     </row>
     <row r="13">
@@ -1093,22 +1093,22 @@
         </is>
       </c>
       <c r="B13" s="20" t="n">
-        <v>1675.8</v>
+        <v>1468.5</v>
       </c>
       <c r="C13" s="17" t="n">
-        <v>1660.6</v>
+        <v>1452.6</v>
       </c>
       <c r="D13" s="7" t="n">
-        <v>1673.8</v>
+        <v>1465.2</v>
       </c>
       <c r="E13" s="30" t="n">
-        <v>1673.6</v>
+        <v>1466.1</v>
       </c>
       <c r="F13" s="9" t="n">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="G13" s="5" t="n">
-        <v>1663.1</v>
+        <v>1465.1</v>
       </c>
     </row>
     <row r="14">
@@ -1118,22 +1118,22 @@
         </is>
       </c>
       <c r="B14" s="20" t="n">
-        <v>1949.9</v>
+        <v>956.3</v>
       </c>
       <c r="C14" s="17" t="n">
-        <v>1926.9</v>
+        <v>940</v>
       </c>
       <c r="D14" s="7" t="n">
-        <v>1940.3</v>
+        <v>953.95</v>
       </c>
       <c r="E14" s="30" t="n">
-        <v>1940.2</v>
+        <v>954.45</v>
       </c>
       <c r="F14" s="9" t="n">
-        <v>54</v>
+        <v>160</v>
       </c>
       <c r="G14" s="5" t="n">
-        <v>1943.2</v>
+        <v>940.75</v>
       </c>
     </row>
     <row r="15">
@@ -1143,22 +1143,22 @@
         </is>
       </c>
       <c r="B15" s="20" t="n">
-        <v>669.7</v>
+        <v>744</v>
       </c>
       <c r="C15" s="17" t="n">
-        <v>654.65</v>
+        <v>725.1</v>
       </c>
       <c r="D15" s="7" t="n">
-        <v>661</v>
+        <v>742.7</v>
       </c>
       <c r="E15" s="30" t="n">
-        <v>661.45</v>
+        <v>742.95</v>
       </c>
       <c r="F15" s="9" t="n">
-        <v>68</v>
+        <v>89</v>
       </c>
       <c r="G15" s="5" t="n">
-        <v>659.25</v>
+        <v>731.25</v>
       </c>
     </row>
     <row r="16">
@@ -1168,22 +1168,22 @@
         </is>
       </c>
       <c r="B16" s="20" t="n">
-        <v>1471.6</v>
+        <v>1400</v>
       </c>
       <c r="C16" s="17" t="n">
-        <v>1455</v>
+        <v>1385.3</v>
       </c>
       <c r="D16" s="7" t="n">
-        <v>1460.5</v>
+        <v>1396.6</v>
       </c>
       <c r="E16" s="30" t="n">
-        <v>1460.6</v>
+        <v>1397</v>
       </c>
       <c r="F16" s="9" t="n">
-        <v>56</v>
+        <v>98</v>
       </c>
       <c r="G16" s="5" t="n">
-        <v>1466.2</v>
+        <v>1385.6</v>
       </c>
     </row>
     <row r="17">
@@ -1193,22 +1193,22 @@
         </is>
       </c>
       <c r="B17" s="20" t="n">
-        <v>802</v>
+        <v>769</v>
       </c>
       <c r="C17" s="17" t="n">
-        <v>790.75</v>
+        <v>754.1</v>
       </c>
       <c r="D17" s="7" t="n">
-        <v>800.75</v>
+        <v>767.8</v>
       </c>
       <c r="E17" s="30" t="n">
-        <v>800.1</v>
+        <v>768.1</v>
       </c>
       <c r="F17" s="9" t="n">
-        <v>53</v>
+        <v>19</v>
       </c>
       <c r="G17" s="5" t="n">
-        <v>797.75</v>
+        <v>755.35</v>
       </c>
     </row>
     <row r="18">
@@ -1218,22 +1218,22 @@
         </is>
       </c>
       <c r="B18" s="20" t="n">
-        <v>1583.8</v>
+        <v>1489.8</v>
       </c>
       <c r="C18" s="17" t="n">
-        <v>1571.8</v>
+        <v>1473</v>
       </c>
       <c r="D18" s="7" t="n">
-        <v>1582</v>
+        <v>1480</v>
       </c>
       <c r="E18" s="30" t="n">
-        <v>1580.5</v>
+        <v>1479.1</v>
       </c>
       <c r="F18" s="9" t="n">
-        <v>31</v>
+        <v>46</v>
       </c>
       <c r="G18" s="5" t="n">
-        <v>1574.3</v>
+        <v>1486.4</v>
       </c>
     </row>
     <row r="19">
@@ -1243,22 +1243,22 @@
         </is>
       </c>
       <c r="B19" s="20" t="n">
-        <v>969.8</v>
+        <v>1030</v>
       </c>
       <c r="C19" s="17" t="n">
-        <v>953.15</v>
+        <v>992.1</v>
       </c>
       <c r="D19" s="7" t="n">
-        <v>954</v>
+        <v>1028.5</v>
       </c>
       <c r="E19" s="30" t="n">
-        <v>954.8</v>
+        <v>1028.35</v>
       </c>
       <c r="F19" s="9" t="n">
-        <v>13</v>
+        <v>45</v>
       </c>
       <c r="G19" s="5" t="n">
-        <v>962.3</v>
+        <v>1000.5</v>
       </c>
     </row>
     <row r="20">
@@ -1268,22 +1268,22 @@
         </is>
       </c>
       <c r="B20" s="20" t="n">
-        <v>605.5</v>
+        <v>559.8</v>
       </c>
       <c r="C20" s="17" t="n">
-        <v>597.05</v>
+        <v>555.65</v>
       </c>
       <c r="D20" s="7" t="n">
-        <v>603</v>
+        <v>557.45</v>
       </c>
       <c r="E20" s="30" t="n">
-        <v>603.35</v>
+        <v>557.1</v>
       </c>
       <c r="F20" s="9" t="n">
-        <v>23</v>
+        <v>6</v>
       </c>
       <c r="G20" s="5" t="n">
-        <v>600.6</v>
+        <v>556.45</v>
       </c>
     </row>
     <row r="21">
@@ -1293,22 +1293,22 @@
         </is>
       </c>
       <c r="B21" s="20" t="n">
-        <v>3101</v>
+        <v>3292.5</v>
       </c>
       <c r="C21" s="17" t="n">
-        <v>3065</v>
+        <v>3232.8</v>
       </c>
       <c r="D21" s="7" t="n">
-        <v>3075</v>
+        <v>3288</v>
       </c>
       <c r="E21" s="30" t="n">
-        <v>3080.2</v>
+        <v>3286</v>
       </c>
       <c r="F21" s="9" t="n">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="G21" s="5" t="n">
-        <v>3091.2</v>
+        <v>3256.9</v>
       </c>
     </row>
     <row r="22">
@@ -1318,22 +1318,22 @@
         </is>
       </c>
       <c r="B22" s="20" t="n">
-        <v>259.4</v>
+        <v>262.9</v>
       </c>
       <c r="C22" s="17" t="n">
-        <v>255.65</v>
+        <v>259.35</v>
       </c>
       <c r="D22" s="7" t="n">
-        <v>256.65</v>
+        <v>259.8</v>
       </c>
       <c r="E22" s="30" t="n">
-        <v>256.5</v>
+        <v>259.7</v>
       </c>
       <c r="F22" s="9" t="n">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="G22" s="5" t="n">
-        <v>258.25</v>
+        <v>259.8</v>
       </c>
     </row>
     <row r="23">
@@ -1343,22 +1343,22 @@
         </is>
       </c>
       <c r="B23" s="20" t="n">
-        <v>349.2</v>
+        <v>337.05</v>
       </c>
       <c r="C23" s="17" t="n">
-        <v>342.55</v>
+        <v>333.5</v>
       </c>
       <c r="D23" s="7" t="n">
-        <v>343.3</v>
+        <v>334.5</v>
       </c>
       <c r="E23" s="30" t="n">
-        <v>343.5</v>
+        <v>334.25</v>
       </c>
       <c r="F23" s="9" t="n">
-        <v>166</v>
+        <v>107</v>
       </c>
       <c r="G23" s="5" t="n">
-        <v>348.9</v>
+        <v>336.85</v>
       </c>
     </row>
     <row r="24">
@@ -1368,22 +1368,22 @@
         </is>
       </c>
       <c r="B24" s="20" t="n">
-        <v>1441</v>
+        <v>1376.5</v>
       </c>
       <c r="C24" s="17" t="n">
-        <v>1433</v>
+        <v>1363.2</v>
       </c>
       <c r="D24" s="7" t="n">
-        <v>1435.9</v>
+        <v>1372</v>
       </c>
       <c r="E24" s="30" t="n">
-        <v>1434.8</v>
+        <v>1372.6</v>
       </c>
       <c r="F24" s="9" t="n">
-        <v>48</v>
+        <v>78</v>
       </c>
       <c r="G24" s="5" t="n">
-        <v>1435.7</v>
+        <v>1365.2</v>
       </c>
     </row>
     <row r="25">
@@ -1393,22 +1393,22 @@
         </is>
       </c>
       <c r="B25" s="20" t="n">
-        <v>796.5</v>
+        <v>813.3</v>
       </c>
       <c r="C25" s="17" t="n">
-        <v>789.2</v>
+        <v>806.5</v>
       </c>
       <c r="D25" s="7" t="n">
-        <v>794.15</v>
+        <v>813</v>
       </c>
       <c r="E25" s="30" t="n">
-        <v>794.4</v>
+        <v>812.15</v>
       </c>
       <c r="F25" s="9" t="n">
-        <v>49</v>
+        <v>42</v>
       </c>
       <c r="G25" s="5" t="n">
-        <v>795.7</v>
+        <v>806.6</v>
       </c>
     </row>
     <row r="26">
@@ -1418,22 +1418,22 @@
         </is>
       </c>
       <c r="B26" s="20" t="n">
-        <v>636.75</v>
+        <v>569.95</v>
       </c>
       <c r="C26" s="17" t="n">
-        <v>629.3</v>
+        <v>559.35</v>
       </c>
       <c r="D26" s="7" t="n">
-        <v>633.7</v>
+        <v>561.45</v>
       </c>
       <c r="E26" s="30" t="n">
-        <v>633.55</v>
+        <v>561.3</v>
       </c>
       <c r="F26" s="9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G26" s="5" t="n">
-        <v>636.15</v>
+        <v>566.5</v>
       </c>
     </row>
     <row r="27">
@@ -1443,22 +1443,22 @@
         </is>
       </c>
       <c r="B27" s="20" t="n">
-        <v>886.7</v>
+        <v>942.35</v>
       </c>
       <c r="C27" s="17" t="n">
-        <v>871.05</v>
+        <v>931.1</v>
       </c>
       <c r="D27" s="7" t="n">
-        <v>881.5</v>
+        <v>939.8</v>
       </c>
       <c r="E27" s="30" t="n">
-        <v>881.85</v>
+        <v>939.2</v>
       </c>
       <c r="F27" s="9" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="G27" s="5" t="n">
-        <v>878.8</v>
+        <v>935.85</v>
       </c>
     </row>
     <row r="28">
@@ -1468,22 +1468,22 @@
         </is>
       </c>
       <c r="B28" s="20" t="n">
-        <v>738</v>
+        <v>693.45</v>
       </c>
       <c r="C28" s="17" t="n">
-        <v>726.5</v>
+        <v>685.7</v>
       </c>
       <c r="D28" s="7" t="n">
-        <v>729.2</v>
+        <v>691.8</v>
       </c>
       <c r="E28" s="30" t="n">
-        <v>729</v>
+        <v>692.05</v>
       </c>
       <c r="F28" s="9" t="n">
-        <v>130</v>
+        <v>60</v>
       </c>
       <c r="G28" s="5" t="n">
-        <v>727.95</v>
+        <v>686.05</v>
       </c>
     </row>
     <row r="29" ht="18" customHeight="1">
@@ -1493,22 +1493,22 @@
         </is>
       </c>
       <c r="B29" s="20" t="n">
-        <v>406</v>
+        <v>389.7</v>
       </c>
       <c r="C29" s="17" t="n">
-        <v>400.6</v>
+        <v>386.2</v>
       </c>
       <c r="D29" s="7" t="n">
-        <v>401.8</v>
+        <v>389</v>
       </c>
       <c r="E29" s="30" t="n">
-        <v>402.6</v>
+        <v>389.15</v>
       </c>
       <c r="F29" s="22" t="n">
-        <v>59</v>
+        <v>26</v>
       </c>
       <c r="G29" s="23" t="n">
-        <v>404.05</v>
+        <v>387.25</v>
       </c>
       <c r="H29" s="33" t="n"/>
     </row>
@@ -1519,22 +1519,22 @@
         </is>
       </c>
       <c r="B30" s="21" t="n">
-        <v>165.55</v>
+        <v>168</v>
       </c>
       <c r="C30" s="18" t="n">
-        <v>162.05</v>
+        <v>160.79</v>
       </c>
       <c r="D30" s="11" t="n">
-        <v>162.37</v>
+        <v>167.83</v>
       </c>
       <c r="E30" s="31" t="n">
-        <v>162.51</v>
+        <v>167.85</v>
       </c>
       <c r="F30" s="24" t="n">
-        <v>255</v>
+        <v>823</v>
       </c>
       <c r="G30" s="24" t="n">
-        <v>163.71</v>
+        <v>161.96</v>
       </c>
     </row>
     <row r="31" ht="15.75" customHeight="1" thickBot="1">
@@ -1544,22 +1544,22 @@
         </is>
       </c>
       <c r="B31" s="21" t="n">
-        <v>11812</v>
+        <v>12770</v>
       </c>
       <c r="C31" s="18" t="n">
-        <v>11645</v>
+        <v>12676</v>
       </c>
       <c r="D31" s="25" t="n">
-        <v>11676</v>
+        <v>12702</v>
       </c>
       <c r="E31" s="32" t="n">
-        <v>11689</v>
+        <v>12733</v>
       </c>
       <c r="F31" s="26" t="n">
         <v>1</v>
       </c>
       <c r="G31" s="27" t="n">
-        <v>11805</v>
+        <v>12704</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fixed 15 min cash issue
</commit_message>
<xml_diff>
--- a/cash high low.xlsx
+++ b/cash high low.xlsx
@@ -818,22 +818,22 @@
         </is>
       </c>
       <c r="B2" s="19" t="n">
-        <v>385.1</v>
+        <v>383.05</v>
       </c>
       <c r="C2" s="16" t="n">
-        <v>378.9</v>
+        <v>376.55</v>
       </c>
       <c r="D2" s="6" t="n">
-        <v>380.9</v>
+        <v>377.5</v>
       </c>
       <c r="E2" s="29" t="n">
-        <v>380.8</v>
+        <v>377.45</v>
       </c>
       <c r="F2" s="8" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>385</v>
+        <v>380.35</v>
       </c>
     </row>
     <row r="3">
@@ -843,22 +843,22 @@
         </is>
       </c>
       <c r="B3" s="19" t="n">
-        <v>2311.5</v>
+        <v>2597</v>
       </c>
       <c r="C3" s="16" t="n">
-        <v>2275</v>
+        <v>2562.6</v>
       </c>
       <c r="D3" s="6" t="n">
-        <v>2280</v>
+        <v>2573</v>
       </c>
       <c r="E3" s="29" t="n">
-        <v>2278.8</v>
+        <v>2573.5</v>
       </c>
       <c r="F3" s="8" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G3" s="4" t="n">
-        <v>2300.1</v>
+        <v>2596.8</v>
       </c>
     </row>
     <row r="4">
@@ -868,22 +868,22 @@
         </is>
       </c>
       <c r="B4" s="20" t="n">
-        <v>497.8</v>
+        <v>479</v>
       </c>
       <c r="C4" s="17" t="n">
-        <v>481.05</v>
+        <v>470.4</v>
       </c>
       <c r="D4" s="7" t="n">
-        <v>485.5</v>
+        <v>474.45</v>
       </c>
       <c r="E4" s="30" t="n">
-        <v>485.5</v>
+        <v>474.7</v>
       </c>
       <c r="F4" s="9" t="n">
-        <v>25</v>
+        <v>7</v>
       </c>
       <c r="G4" s="5" t="n">
-        <v>492.85</v>
+        <v>474</v>
       </c>
     </row>
     <row r="5">
@@ -893,22 +893,22 @@
         </is>
       </c>
       <c r="B5" s="20" t="n">
-        <v>2033.8</v>
+        <v>2042.2</v>
       </c>
       <c r="C5" s="17" t="n">
-        <v>2000</v>
+        <v>2012.1</v>
       </c>
       <c r="D5" s="7" t="n">
-        <v>2003</v>
+        <v>2031.1</v>
       </c>
       <c r="E5" s="30" t="n">
-        <v>2002.2</v>
+        <v>2033.2</v>
       </c>
       <c r="F5" s="9" t="n">
-        <v>24</v>
+        <v>8</v>
       </c>
       <c r="G5" s="5" t="n">
-        <v>2015.9</v>
+        <v>2015.7</v>
       </c>
     </row>
     <row r="6">
@@ -918,22 +918,22 @@
         </is>
       </c>
       <c r="B6" s="20" t="n">
-        <v>948</v>
+        <v>1023</v>
       </c>
       <c r="C6" s="17" t="n">
-        <v>928</v>
+        <v>1003.05</v>
       </c>
       <c r="D6" s="7" t="n">
-        <v>933.05</v>
+        <v>1010</v>
       </c>
       <c r="E6" s="30" t="n">
-        <v>934.75</v>
+        <v>1008.9</v>
       </c>
       <c r="F6" s="9" t="n">
-        <v>217</v>
+        <v>92</v>
       </c>
       <c r="G6" s="5" t="n">
-        <v>940.15</v>
+        <v>1003.05</v>
       </c>
     </row>
     <row r="7">
@@ -943,22 +943,22 @@
         </is>
       </c>
       <c r="B7" s="20" t="n">
-        <v>165.35</v>
+        <v>166.58</v>
       </c>
       <c r="C7" s="17" t="n">
-        <v>162.01</v>
+        <v>164.36</v>
       </c>
       <c r="D7" s="7" t="n">
-        <v>162.7</v>
+        <v>165.21</v>
       </c>
       <c r="E7" s="30" t="n">
-        <v>162.48</v>
+        <v>164.79</v>
       </c>
       <c r="F7" s="9" t="n">
-        <v>22</v>
+        <v>62</v>
       </c>
       <c r="G7" s="5" t="n">
-        <v>164.87</v>
+        <v>165.44</v>
       </c>
     </row>
     <row r="8">
@@ -968,22 +968,22 @@
         </is>
       </c>
       <c r="B8" s="20" t="n">
-        <v>238.88</v>
+        <v>269.3</v>
       </c>
       <c r="C8" s="17" t="n">
-        <v>233.57</v>
+        <v>265.4</v>
       </c>
       <c r="D8" s="7" t="n">
-        <v>234.13</v>
+        <v>265.9</v>
       </c>
       <c r="E8" s="30" t="n">
-        <v>233.94</v>
+        <v>266.6</v>
       </c>
       <c r="F8" s="9" t="n">
-        <v>40</v>
+        <v>139</v>
       </c>
       <c r="G8" s="5" t="n">
-        <v>238.7</v>
+        <v>267.8</v>
       </c>
     </row>
     <row r="9">
@@ -993,22 +993,22 @@
         </is>
       </c>
       <c r="B9" s="20" t="n">
-        <v>392.1</v>
+        <v>383.3</v>
       </c>
       <c r="C9" s="17" t="n">
-        <v>385.7</v>
+        <v>379.95</v>
       </c>
       <c r="D9" s="7" t="n">
-        <v>391.25</v>
+        <v>382.3</v>
       </c>
       <c r="E9" s="30" t="n">
-        <v>391.45</v>
+        <v>381.9</v>
       </c>
       <c r="F9" s="9" t="n">
-        <v>55</v>
+        <v>70</v>
       </c>
       <c r="G9" s="5" t="n">
-        <v>386.4</v>
+        <v>383.05</v>
       </c>
     </row>
     <row r="10">
@@ -1018,22 +1018,22 @@
         </is>
       </c>
       <c r="B10" s="20" t="n">
-        <v>777.3</v>
+        <v>736.4</v>
       </c>
       <c r="C10" s="17" t="n">
-        <v>755.9</v>
+        <v>722.25</v>
       </c>
       <c r="D10" s="7" t="n">
-        <v>758.5</v>
+        <v>735.95</v>
       </c>
       <c r="E10" s="30" t="n">
-        <v>758.1</v>
+        <v>735.25</v>
       </c>
       <c r="F10" s="9" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G10" s="5" t="n">
-        <v>765.35</v>
+        <v>726.6</v>
       </c>
     </row>
     <row r="11">
@@ -1043,22 +1043,22 @@
         </is>
       </c>
       <c r="B11" s="20" t="n">
-        <v>6611</v>
+        <v>6948</v>
       </c>
       <c r="C11" s="17" t="n">
-        <v>6411.5</v>
+        <v>6865</v>
       </c>
       <c r="D11" s="7" t="n">
-        <v>6431</v>
+        <v>6876</v>
       </c>
       <c r="E11" s="30" t="n">
-        <v>6425</v>
+        <v>6880</v>
       </c>
       <c r="F11" s="9" t="n">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="G11" s="5" t="n">
-        <v>6580</v>
+        <v>6927</v>
       </c>
     </row>
     <row r="12">
@@ -1068,22 +1068,22 @@
         </is>
       </c>
       <c r="B12" s="20" t="n">
-        <v>193.89</v>
+        <v>194.09</v>
       </c>
       <c r="C12" s="17" t="n">
-        <v>188.4</v>
+        <v>192.16</v>
       </c>
       <c r="D12" s="7" t="n">
-        <v>190.32</v>
+        <v>193.75</v>
       </c>
       <c r="E12" s="30" t="n">
-        <v>189.9</v>
+        <v>193.66</v>
       </c>
       <c r="F12" s="9" t="n">
-        <v>77</v>
+        <v>50</v>
       </c>
       <c r="G12" s="5" t="n">
-        <v>193.7</v>
+        <v>192.77</v>
       </c>
     </row>
     <row r="13">
@@ -1093,22 +1093,22 @@
         </is>
       </c>
       <c r="B13" s="20" t="n">
-        <v>1465.4</v>
+        <v>1421</v>
       </c>
       <c r="C13" s="17" t="n">
-        <v>1440.9</v>
+        <v>1396</v>
       </c>
       <c r="D13" s="7" t="n">
-        <v>1444.2</v>
+        <v>1416.9</v>
       </c>
       <c r="E13" s="30" t="n">
-        <v>1443.3</v>
+        <v>1417.7</v>
       </c>
       <c r="F13" s="9" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="G13" s="5" t="n">
-        <v>1460.9</v>
+        <v>1397.2</v>
       </c>
     </row>
     <row r="14">
@@ -1118,22 +1118,22 @@
         </is>
       </c>
       <c r="B14" s="20" t="n">
-        <v>965.7</v>
+        <v>977.4</v>
       </c>
       <c r="C14" s="17" t="n">
-        <v>956.25</v>
+        <v>962</v>
       </c>
       <c r="D14" s="7" t="n">
-        <v>960.95</v>
+        <v>973.9</v>
       </c>
       <c r="E14" s="30" t="n">
-        <v>961.25</v>
+        <v>973.45</v>
       </c>
       <c r="F14" s="9" t="n">
-        <v>134</v>
+        <v>185</v>
       </c>
       <c r="G14" s="5" t="n">
-        <v>957.5</v>
+        <v>967.15</v>
       </c>
     </row>
     <row r="15">
@@ -1143,22 +1143,22 @@
         </is>
       </c>
       <c r="B15" s="20" t="n">
-        <v>744.9</v>
+        <v>784.95</v>
       </c>
       <c r="C15" s="17" t="n">
-        <v>737.2</v>
+        <v>774.35</v>
       </c>
       <c r="D15" s="7" t="n">
-        <v>738</v>
+        <v>776.5</v>
       </c>
       <c r="E15" s="30" t="n">
-        <v>739.05</v>
+        <v>776.7</v>
       </c>
       <c r="F15" s="9" t="n">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="G15" s="5" t="n">
-        <v>741.45</v>
+        <v>784.1</v>
       </c>
     </row>
     <row r="16">
@@ -1168,22 +1168,22 @@
         </is>
       </c>
       <c r="B16" s="20" t="n">
-        <v>1415.1</v>
+        <v>1372.1</v>
       </c>
       <c r="C16" s="17" t="n">
-        <v>1404</v>
+        <v>1359.1</v>
       </c>
       <c r="D16" s="7" t="n">
-        <v>1408</v>
+        <v>1363.9</v>
       </c>
       <c r="E16" s="30" t="n">
-        <v>1405.5</v>
+        <v>1363.4</v>
       </c>
       <c r="F16" s="9" t="n">
-        <v>76</v>
+        <v>143</v>
       </c>
       <c r="G16" s="5" t="n">
-        <v>1408</v>
+        <v>1369.5</v>
       </c>
     </row>
     <row r="17">
@@ -1193,22 +1193,22 @@
         </is>
       </c>
       <c r="B17" s="20" t="n">
-        <v>765.6</v>
+        <v>755.6</v>
       </c>
       <c r="C17" s="17" t="n">
-        <v>752.85</v>
+        <v>737.3</v>
       </c>
       <c r="D17" s="7" t="n">
-        <v>755</v>
+        <v>741.3</v>
       </c>
       <c r="E17" s="30" t="n">
-        <v>754.85</v>
+        <v>739.3</v>
       </c>
       <c r="F17" s="9" t="n">
-        <v>14</v>
+        <v>51</v>
       </c>
       <c r="G17" s="5" t="n">
-        <v>764.05</v>
+        <v>752.6</v>
       </c>
     </row>
     <row r="18">
@@ -1218,22 +1218,22 @@
         </is>
       </c>
       <c r="B18" s="20" t="n">
-        <v>1477.9</v>
+        <v>1478.8</v>
       </c>
       <c r="C18" s="17" t="n">
-        <v>1460.1</v>
+        <v>1447</v>
       </c>
       <c r="D18" s="7" t="n">
-        <v>1461.5</v>
+        <v>1474.9</v>
       </c>
       <c r="E18" s="30" t="n">
-        <v>1463</v>
+        <v>1476</v>
       </c>
       <c r="F18" s="9" t="n">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="G18" s="5" t="n">
-        <v>1476.8</v>
+        <v>1448</v>
       </c>
     </row>
     <row r="19">
@@ -1243,22 +1243,22 @@
         </is>
       </c>
       <c r="B19" s="20" t="n">
-        <v>1037.4</v>
+        <v>1061.2</v>
       </c>
       <c r="C19" s="17" t="n">
-        <v>1022.25</v>
+        <v>1043.7</v>
       </c>
       <c r="D19" s="7" t="n">
-        <v>1031</v>
+        <v>1050.7</v>
       </c>
       <c r="E19" s="30" t="n">
-        <v>1031.85</v>
+        <v>1055.9</v>
       </c>
       <c r="F19" s="9" t="n">
-        <v>13</v>
+        <v>23</v>
       </c>
       <c r="G19" s="5" t="n">
-        <v>1024.1</v>
+        <v>1051.5</v>
       </c>
     </row>
     <row r="20">
@@ -1268,22 +1268,22 @@
         </is>
       </c>
       <c r="B20" s="20" t="n">
-        <v>562.65</v>
+        <v>579.55</v>
       </c>
       <c r="C20" s="17" t="n">
-        <v>553.15</v>
+        <v>574.4</v>
       </c>
       <c r="D20" s="7" t="n">
-        <v>554.25</v>
+        <v>577</v>
       </c>
       <c r="E20" s="30" t="n">
-        <v>554.3</v>
+        <v>576.85</v>
       </c>
       <c r="F20" s="9" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G20" s="5" t="n">
-        <v>562.65</v>
+        <v>578.6</v>
       </c>
     </row>
     <row r="21">
@@ -1293,22 +1293,22 @@
         </is>
       </c>
       <c r="B21" s="20" t="n">
-        <v>3535</v>
+        <v>3480</v>
       </c>
       <c r="C21" s="17" t="n">
-        <v>3463.4</v>
+        <v>3427.7</v>
       </c>
       <c r="D21" s="7" t="n">
-        <v>3480</v>
+        <v>3476</v>
       </c>
       <c r="E21" s="30" t="n">
-        <v>3481.5</v>
+        <v>3472</v>
       </c>
       <c r="F21" s="9" t="n">
-        <v>76</v>
+        <v>11</v>
       </c>
       <c r="G21" s="5" t="n">
-        <v>3517</v>
+        <v>3445.3</v>
       </c>
     </row>
     <row r="22">
@@ -1318,22 +1318,22 @@
         </is>
       </c>
       <c r="B22" s="20" t="n">
-        <v>265.45</v>
+        <v>284.85</v>
       </c>
       <c r="C22" s="17" t="n">
-        <v>259.45</v>
+        <v>276.95</v>
       </c>
       <c r="D22" s="7" t="n">
-        <v>264.2</v>
+        <v>284</v>
       </c>
       <c r="E22" s="30" t="n">
-        <v>262.9</v>
+        <v>284.15</v>
       </c>
       <c r="F22" s="9" t="n">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="G22" s="5" t="n">
-        <v>262.9</v>
+        <v>278.3</v>
       </c>
     </row>
     <row r="23">
@@ -1343,22 +1343,22 @@
         </is>
       </c>
       <c r="B23" s="20" t="n">
-        <v>334.9</v>
+        <v>340.8</v>
       </c>
       <c r="C23" s="17" t="n">
-        <v>329.3</v>
+        <v>335.65</v>
       </c>
       <c r="D23" s="7" t="n">
-        <v>330.3</v>
+        <v>339.2</v>
       </c>
       <c r="E23" s="30" t="n">
-        <v>330.05</v>
+        <v>339.1</v>
       </c>
       <c r="F23" s="9" t="n">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="G23" s="5" t="n">
-        <v>333.1</v>
+        <v>340.45</v>
       </c>
     </row>
     <row r="24">
@@ -1368,22 +1368,22 @@
         </is>
       </c>
       <c r="B24" s="20" t="n">
-        <v>1369.9</v>
+        <v>1377.4</v>
       </c>
       <c r="C24" s="17" t="n">
-        <v>1357.1</v>
+        <v>1361</v>
       </c>
       <c r="D24" s="7" t="n">
-        <v>1359.1</v>
+        <v>1374.9</v>
       </c>
       <c r="E24" s="30" t="n">
-        <v>1359.3</v>
+        <v>1375</v>
       </c>
       <c r="F24" s="9" t="n">
-        <v>132</v>
+        <v>123</v>
       </c>
       <c r="G24" s="5" t="n">
-        <v>1365.2</v>
+        <v>1363</v>
       </c>
     </row>
     <row r="25">
@@ -1393,22 +1393,22 @@
         </is>
       </c>
       <c r="B25" s="20" t="n">
-        <v>815</v>
+        <v>875.3</v>
       </c>
       <c r="C25" s="17" t="n">
-        <v>808</v>
+        <v>864.8</v>
       </c>
       <c r="D25" s="7" t="n">
-        <v>809.85</v>
+        <v>873.8</v>
       </c>
       <c r="E25" s="30" t="n">
-        <v>809.4</v>
+        <v>874.05</v>
       </c>
       <c r="F25" s="9" t="n">
-        <v>44</v>
+        <v>78</v>
       </c>
       <c r="G25" s="5" t="n">
-        <v>813.7</v>
+        <v>866.5</v>
       </c>
     </row>
     <row r="26">
@@ -1418,22 +1418,22 @@
         </is>
       </c>
       <c r="B26" s="20" t="n">
-        <v>570.6</v>
+        <v>581.4</v>
       </c>
       <c r="C26" s="17" t="n">
-        <v>557.65</v>
+        <v>564.55</v>
       </c>
       <c r="D26" s="7" t="n">
-        <v>559.4</v>
+        <v>576.8</v>
       </c>
       <c r="E26" s="30" t="n">
-        <v>559.8</v>
+        <v>578.7</v>
       </c>
       <c r="F26" s="9" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="G26" s="5" t="n">
-        <v>561.1</v>
+        <v>568.4</v>
       </c>
     </row>
     <row r="27">
@@ -1443,22 +1443,22 @@
         </is>
       </c>
       <c r="B27" s="20" t="n">
-        <v>944.9</v>
+        <v>943.1</v>
       </c>
       <c r="C27" s="17" t="n">
-        <v>933.7</v>
+        <v>924.4</v>
       </c>
       <c r="D27" s="7" t="n">
-        <v>939.8</v>
+        <v>930</v>
       </c>
       <c r="E27" s="30" t="n">
-        <v>938.75</v>
+        <v>926.75</v>
       </c>
       <c r="F27" s="9" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="G27" s="5" t="n">
-        <v>942.95</v>
+        <v>931.5</v>
       </c>
     </row>
     <row r="28">
@@ -1468,22 +1468,22 @@
         </is>
       </c>
       <c r="B28" s="20" t="n">
-        <v>703.5</v>
+        <v>715.45</v>
       </c>
       <c r="C28" s="17" t="n">
-        <v>685.7</v>
+        <v>706</v>
       </c>
       <c r="D28" s="7" t="n">
-        <v>688</v>
+        <v>712.9</v>
       </c>
       <c r="E28" s="30" t="n">
-        <v>687.5</v>
+        <v>712.65</v>
       </c>
       <c r="F28" s="9" t="n">
-        <v>134</v>
+        <v>103</v>
       </c>
       <c r="G28" s="5" t="n">
-        <v>702.4</v>
+        <v>711</v>
       </c>
     </row>
     <row r="29" ht="18" customHeight="1">
@@ -1493,22 +1493,22 @@
         </is>
       </c>
       <c r="B29" s="20" t="n">
-        <v>389</v>
+        <v>396.4</v>
       </c>
       <c r="C29" s="17" t="n">
-        <v>381.75</v>
+        <v>389.3</v>
       </c>
       <c r="D29" s="7" t="n">
-        <v>382.5</v>
+        <v>395.5</v>
       </c>
       <c r="E29" s="30" t="n">
-        <v>382.6</v>
+        <v>395.55</v>
       </c>
       <c r="F29" s="22" t="n">
         <v>41</v>
       </c>
       <c r="G29" s="23" t="n">
-        <v>387.45</v>
+        <v>393.6</v>
       </c>
       <c r="H29" s="33" t="n"/>
     </row>
@@ -1519,22 +1519,22 @@
         </is>
       </c>
       <c r="B30" s="21" t="n">
-        <v>168.35</v>
+        <v>172.16</v>
       </c>
       <c r="C30" s="18" t="n">
-        <v>166.62</v>
+        <v>169.3</v>
       </c>
       <c r="D30" s="11" t="n">
-        <v>166.7</v>
+        <v>170.35</v>
       </c>
       <c r="E30" s="31" t="n">
-        <v>166.81</v>
+        <v>170.06</v>
       </c>
       <c r="F30" s="24" t="n">
-        <v>263</v>
+        <v>214</v>
       </c>
       <c r="G30" s="24" t="n">
-        <v>166.92</v>
+        <v>171.9</v>
       </c>
     </row>
     <row r="31" ht="15.75" customHeight="1" thickBot="1">
@@ -1544,22 +1544,22 @@
         </is>
       </c>
       <c r="B31" s="21" t="n">
-        <v>12937</v>
+        <v>12100</v>
       </c>
       <c r="C31" s="18" t="n">
-        <v>12634</v>
+        <v>11991</v>
       </c>
       <c r="D31" s="25" t="n">
-        <v>12646</v>
+        <v>12073</v>
       </c>
       <c r="E31" s="32" t="n">
-        <v>12651</v>
+        <v>12055</v>
       </c>
       <c r="F31" s="26" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G31" s="27" t="n">
-        <v>12910</v>
+        <v>12018</v>
       </c>
     </row>
   </sheetData>

</xml_diff>